<commit_message>
Added SoMe descriptions to headline artists
</commit_message>
<xml_diff>
--- a/data/lineup-2026.xlsx
+++ b/data/lineup-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pekkos/git/bingsjostamman.se/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0EEFD32-429E-CA4E-9468-72C8E733F782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD32516D-88A2-8A46-9D30-6FECF352663D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23640" yWindow="-25940" windowWidth="38320" windowHeight="25360" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="149">
   <si>
     <t>day</t>
   </si>
@@ -471,6 +471,18 @@
   </si>
   <si>
     <t>Invigningsprogrammets konsert</t>
+  </si>
+  <si>
+    <t>somedescription</t>
+  </si>
+  <si>
+    <t>Orgelspelmannen Merit Hemmingson tar sig an Bingsjömusiken på sitt eget vis och ger Pekkos Pers låtar en ny, elektrisk form.</t>
+  </si>
+  <si>
+    <t>På den finska folkmusikhimlen är Polenta ett åttaarmat musikaliskt vidunder. Ett tätt samspel och öppenhet för influenser utmärker Polentas halsbrytande och svindlande musikanteri och de blandar sin musik med lika delar tradition, förnyelse och spelglädje.</t>
+  </si>
+  <si>
+    <t>Spelmannen Hjort Anders Olsson hyllas med konsert och ny utställning. I toner och ord får vi stifta bekantskap med denna legendariska fiolspelman.</t>
   </si>
 </sst>
 </file>
@@ -878,7 +890,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F23F1BC-D35E-3E42-8F88-5D61ED802479}">
-  <dimension ref="A1:N74"/>
+  <dimension ref="A1:O74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.83203125" bestFit="1" customWidth="1"/>
@@ -892,9 +904,11 @@
     <col min="11" max="11" width="28.6640625" customWidth="1"/>
     <col min="12" max="12" width="43.6640625" style="3" customWidth="1"/>
     <col min="13" max="13" width="33.5" customWidth="1"/>
+    <col min="14" max="14" width="28.5" customWidth="1"/>
+    <col min="15" max="15" width="35.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -937,8 +951,11 @@
       <c r="N1" s="3" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="238" x14ac:dyDescent="0.2">
+      <c r="O1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="238" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -981,8 +998,11 @@
       <c r="N2" s="3" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1011,7 +1031,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1034,7 +1054,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1057,7 +1077,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1083,7 +1103,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1106,7 +1126,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -1135,7 +1155,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="153" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" ht="153" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1178,8 +1198,11 @@
       <c r="N9" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="O9" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -1202,7 +1225,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1231,7 +1254,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1258,7 +1281,7 @@
       </c>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1285,7 +1308,7 @@
       </c>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1312,7 +1335,7 @@
       </c>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1338,7 +1361,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -2622,7 +2645,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>5</v>
       </c>
@@ -2648,7 +2671,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>5</v>
       </c>
@@ -2674,7 +2697,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>5</v>
       </c>
@@ -2700,7 +2723,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>5</v>
       </c>
@@ -2726,7 +2749,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="51" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>5</v>
       </c>
@@ -2755,7 +2778,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="68" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:15" ht="68" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>5</v>
       </c>
@@ -2784,7 +2807,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="85" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:15" ht="85" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>5</v>
       </c>
@@ -2813,7 +2836,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:15" ht="34" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>5</v>
       </c>
@@ -2842,7 +2865,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="221" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:15" ht="221" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>5</v>
       </c>
@@ -2882,8 +2905,11 @@
       <c r="N73" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="74" spans="1:14" ht="68" x14ac:dyDescent="0.2">
+      <c r="O73" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" ht="68" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Update lineup page with all acts
</commit_message>
<xml_diff>
--- a/data/lineup-2026.xlsx
+++ b/data/lineup-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pekkos/git/bingsjostamman.se/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B109847E-B636-F445-B78F-54DBFF037D92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9326573-EB5F-F24F-B9D0-A65CA3051B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="67200" windowHeight="37200" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="155">
   <si>
     <t>day</t>
   </si>
@@ -1672,8 +1672,8 @@
       <c r="H26" t="s">
         <v>10</v>
       </c>
-      <c r="I26">
-        <v>18</v>
+      <c r="I26" t="s">
+        <v>32</v>
       </c>
       <c r="J26" s="3" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Added forgotten Dansladu acts
</commit_message>
<xml_diff>
--- a/data/lineup-2026.xlsx
+++ b/data/lineup-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pekkos/git/bingsjostamman.se/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{494E904B-C493-E04C-A33B-9862C3FDE868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F58694-61E0-9A4A-AA28-10B8F8885256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="39620" windowHeight="34980" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="172">
   <si>
     <t>day</t>
   </si>
@@ -528,6 +528,30 @@
   </si>
   <si>
     <t>2026/osten-med-resten_d0bw6k.jpg</t>
+  </si>
+  <si>
+    <t>Balladdans &amp; Kårebockens trallarlag</t>
+  </si>
+  <si>
+    <t>Saxdalens spelmanslag</t>
+  </si>
+  <si>
+    <t>Floda spelmanslag</t>
+  </si>
+  <si>
+    <t>Avesta spelmanslag</t>
+  </si>
+  <si>
+    <t>Boda spelmanslag</t>
+  </si>
+  <si>
+    <t>Järna spelmanslag</t>
+  </si>
+  <si>
+    <t>Mora spelmanslag</t>
+  </si>
+  <si>
+    <t>Gagnef spelmanslag</t>
   </si>
 </sst>
 </file>
@@ -942,7 +966,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F23F1BC-D35E-3E42-8F88-5D61ED802479}">
-  <dimension ref="A1:O74"/>
+  <dimension ref="A1:O82"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.83203125" bestFit="1" customWidth="1"/>
@@ -3035,6 +3059,214 @@
         <v>127</v>
       </c>
     </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>5</v>
+      </c>
+      <c r="B75" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C75" s="2">
+        <v>0.81944444444444442</v>
+      </c>
+      <c r="D75" t="s">
+        <v>43</v>
+      </c>
+      <c r="E75" t="s">
+        <v>24</v>
+      </c>
+      <c r="G75" t="s">
+        <v>33</v>
+      </c>
+      <c r="H75" t="s">
+        <v>164</v>
+      </c>
+      <c r="I75">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>5</v>
+      </c>
+      <c r="B76" s="2">
+        <v>0.81944444444444442</v>
+      </c>
+      <c r="C76" s="2">
+        <v>0.84722222222222221</v>
+      </c>
+      <c r="D76" t="s">
+        <v>43</v>
+      </c>
+      <c r="E76" t="s">
+        <v>24</v>
+      </c>
+      <c r="G76" t="s">
+        <v>33</v>
+      </c>
+      <c r="H76" t="s">
+        <v>165</v>
+      </c>
+      <c r="I76">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>5</v>
+      </c>
+      <c r="B77" s="2">
+        <v>0.84722222222222221</v>
+      </c>
+      <c r="C77" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="D77" t="s">
+        <v>43</v>
+      </c>
+      <c r="E77" t="s">
+        <v>24</v>
+      </c>
+      <c r="G77" t="s">
+        <v>33</v>
+      </c>
+      <c r="H77" t="s">
+        <v>166</v>
+      </c>
+      <c r="I77">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>5</v>
+      </c>
+      <c r="B78" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C78" s="2">
+        <v>0.90277777777777779</v>
+      </c>
+      <c r="D78" t="s">
+        <v>43</v>
+      </c>
+      <c r="E78" t="s">
+        <v>24</v>
+      </c>
+      <c r="G78" t="s">
+        <v>33</v>
+      </c>
+      <c r="H78" t="s">
+        <v>167</v>
+      </c>
+      <c r="I78">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>5</v>
+      </c>
+      <c r="B79" s="2">
+        <v>0.90277777777777779</v>
+      </c>
+      <c r="C79" s="2">
+        <v>0.93055555555555558</v>
+      </c>
+      <c r="D79" t="s">
+        <v>43</v>
+      </c>
+      <c r="E79" t="s">
+        <v>24</v>
+      </c>
+      <c r="G79" t="s">
+        <v>33</v>
+      </c>
+      <c r="H79" t="s">
+        <v>168</v>
+      </c>
+      <c r="I79">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>5</v>
+      </c>
+      <c r="B80" s="2">
+        <v>0.93055555555555558</v>
+      </c>
+      <c r="C80" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="D80" t="s">
+        <v>43</v>
+      </c>
+      <c r="E80" t="s">
+        <v>24</v>
+      </c>
+      <c r="G80" t="s">
+        <v>33</v>
+      </c>
+      <c r="H80" t="s">
+        <v>169</v>
+      </c>
+      <c r="I80">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>5</v>
+      </c>
+      <c r="B81" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="C81" s="2">
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="D81" t="s">
+        <v>43</v>
+      </c>
+      <c r="E81" t="s">
+        <v>24</v>
+      </c>
+      <c r="G81" t="s">
+        <v>33</v>
+      </c>
+      <c r="H81" t="s">
+        <v>170</v>
+      </c>
+      <c r="I81">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>5</v>
+      </c>
+      <c r="B82" s="2">
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="C82" s="2">
+        <v>1.3888888888888888E-2</v>
+      </c>
+      <c r="D82" t="s">
+        <v>43</v>
+      </c>
+      <c r="E82" t="s">
+        <v>24</v>
+      </c>
+      <c r="G82" t="s">
+        <v>33</v>
+      </c>
+      <c r="H82" t="s">
+        <v>171</v>
+      </c>
+      <c r="I82">
+        <v>69</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Added day program pages and restructured some components
</commit_message>
<xml_diff>
--- a/data/lineup-2026.xlsx
+++ b/data/lineup-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pekkos/git/bingsjostamman.se/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F58694-61E0-9A4A-AA28-10B8F8885256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B9C99E8-D237-7E40-8991-A6E91E26ADF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="39620" windowHeight="34980" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="173">
   <si>
     <t>day</t>
   </si>
@@ -182,12 +182,6 @@
     <t>upplev</t>
   </si>
   <si>
-    <t>Bystugan</t>
-  </si>
-  <si>
-    <t>Lanthandeln</t>
-  </si>
-  <si>
     <t>Till Bingsjöbergets topp</t>
   </si>
   <si>
@@ -197,15 +191,9 @@
     <t xml:space="preserve">Upplev en stilla morgonvandring med vallmusiker som blåser horn, kular och delar berättelser längs den 4 km långa stigen tur och retur. Ta med matsöck eller köp smörgåspaket. Samling vid bystugan. </t>
   </si>
   <si>
-    <t>Spelmansgårdar i Bingjö by–Hjort, Junkas, Nylands och Slunk, kända för spelmän och låtar. Följ med på en guidad byvandring, se gårdarna och hör berättelserna. Samling vid lanthandeln där Peo Österholm och Siv Tillsjö är guider.</t>
-  </si>
-  <si>
     <t>Danielsgården</t>
   </si>
   <si>
-    <t>Upplev Winter Carl Hanssons (1777–1805) unika dalmålningar. Guidade visningar. Biljetter från kl. 15 på Danielsgården. Pris 50 kr (endast kontant). Servering 15–19.</t>
-  </si>
-  <si>
     <t>Dräktakuten</t>
   </si>
   <si>
@@ -230,9 +218,6 @@
     <t>Levande Ladan</t>
   </si>
   <si>
-    <t>Upplev en stunds stillhet med sångsektionen i Dalarnas Spelmansförbund. Dela med dig av dina favotirvisor, sjung eller sit med och lyssna. Värd är Lissman Gunnar Turesson.</t>
-  </si>
-  <si>
     <t>Älvdalens spelmanslag</t>
   </si>
   <si>
@@ -398,9 +383,6 @@
     <t>Dansa folkdans (från 10 år)</t>
   </si>
   <si>
-    <t>En skog avt toner</t>
-  </si>
-  <si>
     <t>Bingsjös längsta långdans?</t>
   </si>
   <si>
@@ -552,6 +534,27 @@
   </si>
   <si>
     <t>Gagnef spelmanslag</t>
+  </si>
+  <si>
+    <t>En skog av toner</t>
+  </si>
+  <si>
+    <t>Spelmansgårdar i Bingjö by; Hjort, Junkas, Päkkos, Nylands och Slunk, kända för spelmän och låtar. Följ med på en guidad byvandring, se gårdarna och hör berättelserna. Samling vid lanthandeln där Peo Österholm och Siv Tillsjö är guider.</t>
+  </si>
+  <si>
+    <t>Bingsjö</t>
+  </si>
+  <si>
+    <t>Upplev en stunds stillhet med sångsektionen i Dalarnas Spelmansförbund. Dela med dig av dina favotirvisor, sjung eller sitt med och lyssna. Värd är Lissman Gunnar Turesson.</t>
+  </si>
+  <si>
+    <t>Servering</t>
+  </si>
+  <si>
+    <t>Upplev Winter Carl Hanssons (1777–1805) unika dalmålningar. Guidade visningar. Biljetter från kl. 15 på Danielsgården. Pris 50 kr (endast kontant).</t>
+  </si>
+  <si>
+    <t>Servering av fika alldeles runt knuten på Danielsgården.</t>
   </si>
 </sst>
 </file>
@@ -966,7 +969,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F23F1BC-D35E-3E42-8F88-5D61ED802479}">
-  <dimension ref="A1:O82"/>
+  <dimension ref="A1:O83"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.83203125" bestFit="1" customWidth="1"/>
@@ -1025,10 +1028,10 @@
         <v>3</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="O1" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="238" x14ac:dyDescent="0.2">
@@ -1054,28 +1057,28 @@
         <v>33</v>
       </c>
       <c r="H2" t="s">
+        <v>130</v>
+      </c>
+      <c r="I2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="I2" t="s">
-        <v>86</v>
-      </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L2" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
+        <v>125</v>
+      </c>
+      <c r="N2" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="L2" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="M2" t="s">
-        <v>131</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>135</v>
-      </c>
       <c r="O2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
@@ -1098,16 +1101,16 @@
         <v>33</v>
       </c>
       <c r="H3" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="I3" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="K3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="34" x14ac:dyDescent="0.2">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1121,14 +1124,14 @@
         <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>73</v>
+        <v>68</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>82</v>
       </c>
       <c r="I4">
         <v>1</v>
       </c>
-      <c r="J4" s="3" t="s">
-        <v>87</v>
-      </c>
     </row>
     <row r="5" spans="1:15" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -1144,14 +1147,14 @@
         <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>73</v>
+        <v>68</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>83</v>
       </c>
       <c r="I5">
         <v>2</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>88</v>
-      </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -1167,7 +1170,7 @@
         <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G6" t="s">
         <v>33</v>
@@ -1176,10 +1179,10 @@
         <v>17</v>
       </c>
       <c r="I6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" ht="17" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1193,14 +1196,14 @@
         <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>73</v>
+        <v>68</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>84</v>
       </c>
       <c r="I7">
         <v>3</v>
       </c>
-      <c r="J7" s="3" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="8" spans="1:15" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -1216,19 +1219,19 @@
         <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G8" t="s">
         <v>33</v>
       </c>
       <c r="H8" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="I8" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="153" x14ac:dyDescent="0.2">
@@ -1245,7 +1248,7 @@
         <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F9" t="s">
         <v>29</v>
@@ -1257,25 +1260,25 @@
         <v>39</v>
       </c>
       <c r="I9" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>40</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="M9" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="N9" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="O9" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="17" x14ac:dyDescent="0.2">
@@ -1292,13 +1295,13 @@
         <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>73</v>
+        <v>68</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="I10">
         <v>4</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="17" x14ac:dyDescent="0.2">
@@ -1330,7 +1333,7 @@
         <v>41</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -1437,7 +1440,7 @@
         <v>39</v>
       </c>
       <c r="I15" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
@@ -1514,7 +1517,7 @@
         <v>46</v>
       </c>
       <c r="I18" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="J18" s="4"/>
       <c r="K18" s="1"/>
@@ -1530,19 +1533,19 @@
         <v>0.5</v>
       </c>
       <c r="D19" t="s">
-        <v>48</v>
+        <v>168</v>
       </c>
       <c r="E19" t="s">
         <v>47</v>
       </c>
       <c r="H19" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I19">
         <v>11</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K19" s="1"/>
     </row>
@@ -1557,23 +1560,23 @@
         <v>0.47916666666666669</v>
       </c>
       <c r="D20" t="s">
-        <v>49</v>
+        <v>168</v>
       </c>
       <c r="E20" t="s">
         <v>47</v>
       </c>
       <c r="H20" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="I20">
         <v>12</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>53</v>
+        <v>167</v>
       </c>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="1:13" ht="68" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" ht="51" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>5</v>
       </c>
@@ -1584,7 +1587,7 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="D21" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E21" t="s">
         <v>47</v>
@@ -1596,85 +1599,85 @@
         <v>13</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" ht="102" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>5</v>
       </c>
       <c r="B22" s="2">
-        <v>0.58333333333333337</v>
+        <v>0.625</v>
       </c>
       <c r="C22" s="2">
-        <v>0.75</v>
+        <v>0.79166666666666663</v>
       </c>
       <c r="D22" t="s">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="E22" t="s">
         <v>47</v>
       </c>
       <c r="H22" t="s">
-        <v>56</v>
+        <v>170</v>
       </c>
       <c r="I22">
+        <v>135</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="102" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="2">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C23" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="D23" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H23" t="s">
+        <v>52</v>
+      </c>
+      <c r="I23">
         <v>14</v>
       </c>
-      <c r="J22" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" ht="68" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" s="2">
+      <c r="J23" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="68" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="2">
         <v>0.45833333333333331</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C24" s="2">
         <v>0.54166666666666663</v>
-      </c>
-      <c r="D23" t="s">
-        <v>18</v>
-      </c>
-      <c r="E23" t="s">
-        <v>58</v>
-      </c>
-      <c r="H23" t="s">
-        <v>59</v>
-      </c>
-      <c r="I23">
-        <v>15</v>
-      </c>
-      <c r="J23" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="51" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" s="2">
-        <v>0.64583333333333337</v>
-      </c>
-      <c r="C24" s="2">
-        <v>0.6875</v>
       </c>
       <c r="D24" t="s">
         <v>18</v>
       </c>
       <c r="E24" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="H24" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I24">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="51" x14ac:dyDescent="0.2">
@@ -1682,57 +1685,51 @@
         <v>5</v>
       </c>
       <c r="B25" s="2">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="C25" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="D25" t="s">
+        <v>18</v>
+      </c>
+      <c r="E25" t="s">
+        <v>54</v>
+      </c>
+      <c r="H25" t="s">
+        <v>57</v>
+      </c>
+      <c r="I25">
+        <v>16</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="68" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" s="2">
         <v>0.85416666666666663</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C26" s="2">
         <v>0.91666666666666663</v>
       </c>
-      <c r="D25" t="s">
-        <v>63</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="D26" t="s">
+        <v>59</v>
+      </c>
+      <c r="E26" t="s">
         <v>26</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H26" t="s">
         <v>15</v>
       </c>
-      <c r="I25">
+      <c r="I26">
         <v>17</v>
       </c>
-      <c r="J25" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" ht="17" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>5</v>
-      </c>
-      <c r="B26" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="C26" s="2">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="D26" t="s">
-        <v>16</v>
-      </c>
-      <c r="E26" t="s">
-        <v>23</v>
-      </c>
-      <c r="G26" t="s">
-        <v>33</v>
-      </c>
-      <c r="H26" t="s">
-        <v>10</v>
-      </c>
-      <c r="I26" t="s">
-        <v>32</v>
-      </c>
       <c r="J26" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="K26" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1740,10 +1737,10 @@
         <v>5</v>
       </c>
       <c r="B27" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C27" s="2">
         <v>0.83333333333333337</v>
-      </c>
-      <c r="C27" s="2">
-        <v>0.875</v>
       </c>
       <c r="D27" t="s">
         <v>16</v>
@@ -1755,13 +1752,16 @@
         <v>33</v>
       </c>
       <c r="H27" t="s">
-        <v>65</v>
-      </c>
-      <c r="I27">
-        <v>19</v>
+        <v>10</v>
+      </c>
+      <c r="I27" t="s">
+        <v>32</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>72</v>
+        <v>34</v>
+      </c>
+      <c r="K27" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1769,10 +1769,10 @@
         <v>5</v>
       </c>
       <c r="B28" s="2">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="C28" s="2">
         <v>0.875</v>
-      </c>
-      <c r="C28" s="2">
-        <v>0.91666666666666696</v>
       </c>
       <c r="D28" t="s">
         <v>16</v>
@@ -1784,19 +1784,13 @@
         <v>33</v>
       </c>
       <c r="H28" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="I28">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="K28" t="s">
-        <v>157</v>
-      </c>
-      <c r="M28" t="s">
-        <v>159</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1804,10 +1798,10 @@
         <v>5</v>
       </c>
       <c r="B29" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C29" s="2">
         <v>0.91666666666666696</v>
-      </c>
-      <c r="C29" s="2">
-        <v>0.95833333333333304</v>
       </c>
       <c r="D29" t="s">
         <v>16</v>
@@ -1819,16 +1813,19 @@
         <v>33</v>
       </c>
       <c r="H29" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="I29">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="K29" t="s">
-        <v>162</v>
+        <v>151</v>
+      </c>
+      <c r="M29" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1836,10 +1833,10 @@
         <v>5</v>
       </c>
       <c r="B30" s="2">
-        <v>0.95833333333333404</v>
+        <v>0.91666666666666696</v>
       </c>
       <c r="C30" s="2">
-        <v>1</v>
+        <v>0.95833333333333304</v>
       </c>
       <c r="D30" t="s">
         <v>16</v>
@@ -1851,36 +1848,45 @@
         <v>33</v>
       </c>
       <c r="H30" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="I30">
+        <v>21</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="K30" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>5</v>
+      </c>
+      <c r="B31" s="2">
+        <v>0.95833333333333404</v>
+      </c>
+      <c r="C31" s="2">
+        <v>1</v>
+      </c>
+      <c r="D31" t="s">
+        <v>16</v>
+      </c>
+      <c r="E31" t="s">
+        <v>23</v>
+      </c>
+      <c r="G31" t="s">
+        <v>33</v>
+      </c>
+      <c r="H31" t="s">
+        <v>63</v>
+      </c>
+      <c r="I31">
         <v>22</v>
       </c>
-      <c r="J30" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>5</v>
-      </c>
-      <c r="B31" s="2">
-        <v>0.625</v>
-      </c>
-      <c r="C31" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D31" t="s">
-        <v>21</v>
-      </c>
-      <c r="E31" t="s">
-        <v>25</v>
-      </c>
-      <c r="H31" t="s">
-        <v>74</v>
-      </c>
-      <c r="I31">
-        <v>23</v>
+      <c r="J31" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
@@ -1888,39 +1894,33 @@
         <v>5</v>
       </c>
       <c r="B32" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="C32" s="2">
         <v>0.79166666666666663</v>
-      </c>
-      <c r="C32" s="2">
-        <v>0.83333333333333337</v>
       </c>
       <c r="D32" t="s">
         <v>21</v>
       </c>
       <c r="E32" t="s">
-        <v>24</v>
-      </c>
-      <c r="G32" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="H32" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="I32">
-        <v>24</v>
-      </c>
-      <c r="K32" t="s">
-        <v>158</v>
+        <v>23</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>5</v>
       </c>
-      <c r="B33" s="6">
+      <c r="B33" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C33" s="2">
         <v>0.83333333333333337</v>
-      </c>
-      <c r="C33" s="2">
-        <v>0.86111111111111116</v>
       </c>
       <c r="D33" t="s">
         <v>21</v>
@@ -1932,21 +1932,24 @@
         <v>33</v>
       </c>
       <c r="H33" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="I33">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="K33" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>5</v>
       </c>
-      <c r="B34" s="2">
+      <c r="B34" s="6">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="C34" s="2">
         <v>0.86111111111111116</v>
-      </c>
-      <c r="C34" s="2">
-        <v>0.90277777777777779</v>
       </c>
       <c r="D34" t="s">
         <v>21</v>
@@ -1958,10 +1961,10 @@
         <v>33</v>
       </c>
       <c r="H34" t="s">
-        <v>82</v>
-      </c>
-      <c r="I34" t="s">
-        <v>84</v>
+        <v>78</v>
+      </c>
+      <c r="I34">
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
@@ -1969,10 +1972,10 @@
         <v>5</v>
       </c>
       <c r="B35" s="2">
+        <v>0.86111111111111116</v>
+      </c>
+      <c r="C35" s="2">
         <v>0.90277777777777779</v>
-      </c>
-      <c r="C35" s="2">
-        <v>0.93055555555555558</v>
       </c>
       <c r="D35" t="s">
         <v>21</v>
@@ -1984,10 +1987,10 @@
         <v>33</v>
       </c>
       <c r="H35" t="s">
-        <v>81</v>
-      </c>
-      <c r="I35">
-        <v>26</v>
+        <v>77</v>
+      </c>
+      <c r="I35" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
@@ -1995,10 +1998,10 @@
         <v>5</v>
       </c>
       <c r="B36" s="2">
+        <v>0.90277777777777779</v>
+      </c>
+      <c r="C36" s="2">
         <v>0.93055555555555558</v>
-      </c>
-      <c r="C36" s="2">
-        <v>0.95833333333333337</v>
       </c>
       <c r="D36" t="s">
         <v>21</v>
@@ -2010,16 +2013,10 @@
         <v>33</v>
       </c>
       <c r="H36" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I36">
-        <v>27</v>
-      </c>
-      <c r="K36" t="s">
-        <v>156</v>
-      </c>
-      <c r="M36" t="s">
-        <v>160</v>
+        <v>26</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
@@ -2027,10 +2024,10 @@
         <v>5</v>
       </c>
       <c r="B37" s="2">
+        <v>0.93055555555555558</v>
+      </c>
+      <c r="C37" s="2">
         <v>0.95833333333333337</v>
-      </c>
-      <c r="C37" s="2">
-        <v>0.98611111111111116</v>
       </c>
       <c r="D37" t="s">
         <v>21</v>
@@ -2042,13 +2039,16 @@
         <v>33</v>
       </c>
       <c r="H37" t="s">
-        <v>79</v>
-      </c>
-      <c r="I37" t="s">
-        <v>32</v>
+        <v>75</v>
+      </c>
+      <c r="I37">
+        <v>27</v>
       </c>
       <c r="K37" t="s">
-        <v>155</v>
+        <v>150</v>
+      </c>
+      <c r="M37" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
@@ -2056,10 +2056,10 @@
         <v>5</v>
       </c>
       <c r="B38" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="C38" s="2">
         <v>0.98611111111111116</v>
-      </c>
-      <c r="C38" s="2">
-        <v>1.3888888888888888E-2</v>
       </c>
       <c r="D38" t="s">
         <v>21</v>
@@ -2071,13 +2071,13 @@
         <v>33</v>
       </c>
       <c r="H38" t="s">
-        <v>78</v>
-      </c>
-      <c r="I38">
-        <v>28</v>
-      </c>
-      <c r="M38" t="s">
-        <v>161</v>
+        <v>74</v>
+      </c>
+      <c r="I38" t="s">
+        <v>32</v>
+      </c>
+      <c r="K38" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
@@ -2085,10 +2085,10 @@
         <v>5</v>
       </c>
       <c r="B39" s="2">
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="C39" s="2">
         <v>1.3888888888888888E-2</v>
-      </c>
-      <c r="C39" s="2">
-        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D39" t="s">
         <v>21</v>
@@ -2100,10 +2100,13 @@
         <v>33</v>
       </c>
       <c r="H39" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I39">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="M39" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
@@ -2111,10 +2114,10 @@
         <v>5</v>
       </c>
       <c r="B40" s="2">
+        <v>1.3888888888888888E-2</v>
+      </c>
+      <c r="C40" s="2">
         <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C40" s="2">
-        <v>6.9444444444444448E-2</v>
       </c>
       <c r="D40" t="s">
         <v>21</v>
@@ -2126,10 +2129,10 @@
         <v>33</v>
       </c>
       <c r="H40" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="I40">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
@@ -2137,28 +2140,25 @@
         <v>5</v>
       </c>
       <c r="B41" s="2">
-        <v>0.79166666666666663</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="C41" s="2">
-        <v>0.8125</v>
+        <v>6.9444444444444448E-2</v>
       </c>
       <c r="D41" t="s">
         <v>21</v>
       </c>
       <c r="E41" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G41" t="s">
         <v>33</v>
       </c>
       <c r="H41" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="I41">
-        <v>31</v>
-      </c>
-      <c r="M41" t="s">
-        <v>151</v>
+        <v>30</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
@@ -2166,13 +2166,13 @@
         <v>5</v>
       </c>
       <c r="B42" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C42" s="2">
         <v>0.8125</v>
       </c>
-      <c r="C42" s="2">
-        <v>0.83333333333333304</v>
-      </c>
       <c r="D42" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E42" t="s">
         <v>25</v>
@@ -2181,22 +2181,24 @@
         <v>33</v>
       </c>
       <c r="H42" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="I42">
-        <v>32</v>
-      </c>
-      <c r="K42" s="1"/>
+        <v>31</v>
+      </c>
+      <c r="M42" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>5</v>
       </c>
       <c r="B43" s="2">
+        <v>0.8125</v>
+      </c>
+      <c r="C43" s="2">
         <v>0.83333333333333304</v>
-      </c>
-      <c r="C43" s="2">
-        <v>0.85416666666666696</v>
       </c>
       <c r="D43" t="s">
         <v>11</v>
@@ -2208,21 +2210,22 @@
         <v>33</v>
       </c>
       <c r="H43" t="s">
-        <v>17</v>
-      </c>
-      <c r="I43" t="s">
-        <v>84</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="I43">
+        <v>32</v>
+      </c>
+      <c r="K43" s="1"/>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>5</v>
       </c>
       <c r="B44" s="2">
+        <v>0.83333333333333304</v>
+      </c>
+      <c r="C44" s="2">
         <v>0.85416666666666696</v>
-      </c>
-      <c r="C44" s="2">
-        <v>0.875</v>
       </c>
       <c r="D44" t="s">
         <v>11</v>
@@ -2230,11 +2233,14 @@
       <c r="E44" t="s">
         <v>25</v>
       </c>
+      <c r="G44" t="s">
+        <v>33</v>
+      </c>
       <c r="H44" t="s">
-        <v>94</v>
-      </c>
-      <c r="I44">
-        <v>33</v>
+        <v>17</v>
+      </c>
+      <c r="I44" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
@@ -2242,10 +2248,10 @@
         <v>5</v>
       </c>
       <c r="B45" s="2">
+        <v>0.85416666666666696</v>
+      </c>
+      <c r="C45" s="2">
         <v>0.875</v>
-      </c>
-      <c r="C45" s="2">
-        <v>0.89583333333333404</v>
       </c>
       <c r="D45" t="s">
         <v>11</v>
@@ -2253,14 +2259,11 @@
       <c r="E45" t="s">
         <v>25</v>
       </c>
-      <c r="G45" t="s">
-        <v>33</v>
-      </c>
       <c r="H45" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="I45">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
@@ -2268,10 +2271,10 @@
         <v>5</v>
       </c>
       <c r="B46" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C46" s="2">
         <v>0.89583333333333404</v>
-      </c>
-      <c r="C46" s="2">
-        <v>0.91666666666666696</v>
       </c>
       <c r="D46" t="s">
         <v>11</v>
@@ -2283,10 +2286,10 @@
         <v>33</v>
       </c>
       <c r="H46" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="I46">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
@@ -2294,10 +2297,10 @@
         <v>5</v>
       </c>
       <c r="B47" s="2">
+        <v>0.89583333333333404</v>
+      </c>
+      <c r="C47" s="2">
         <v>0.91666666666666696</v>
-      </c>
-      <c r="C47" s="2">
-        <v>0.937500000000001</v>
       </c>
       <c r="D47" t="s">
         <v>11</v>
@@ -2309,21 +2312,21 @@
         <v>33</v>
       </c>
       <c r="H47" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="I47">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>5</v>
       </c>
       <c r="B48" s="2">
+        <v>0.91666666666666696</v>
+      </c>
+      <c r="C48" s="2">
         <v>0.937500000000001</v>
-      </c>
-      <c r="C48" s="2">
-        <v>0.95833333333333404</v>
       </c>
       <c r="D48" t="s">
         <v>11</v>
@@ -2335,27 +2338,21 @@
         <v>33</v>
       </c>
       <c r="H48" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="I48">
-        <v>37</v>
-      </c>
-      <c r="L48" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="M48" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>5</v>
       </c>
       <c r="B49" s="2">
+        <v>0.937500000000001</v>
+      </c>
+      <c r="C49" s="2">
         <v>0.95833333333333404</v>
-      </c>
-      <c r="C49" s="2">
-        <v>0.97916666666666696</v>
       </c>
       <c r="D49" t="s">
         <v>11</v>
@@ -2367,10 +2364,16 @@
         <v>33</v>
       </c>
       <c r="H49" t="s">
-        <v>128</v>
+        <v>93</v>
       </c>
       <c r="I49">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="L49" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="M49" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.2">
@@ -2378,10 +2381,10 @@
         <v>5</v>
       </c>
       <c r="B50" s="2">
+        <v>0.95833333333333404</v>
+      </c>
+      <c r="C50" s="2">
         <v>0.97916666666666696</v>
-      </c>
-      <c r="C50" s="2">
-        <v>1</v>
       </c>
       <c r="D50" t="s">
         <v>11</v>
@@ -2393,13 +2396,10 @@
         <v>33</v>
       </c>
       <c r="H50" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="I50">
-        <v>39</v>
-      </c>
-      <c r="M50" t="s">
-        <v>152</v>
+        <v>38</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.2">
@@ -2407,10 +2407,10 @@
         <v>5</v>
       </c>
       <c r="B51" s="2">
+        <v>0.97916666666666696</v>
+      </c>
+      <c r="C51" s="2">
         <v>1</v>
-      </c>
-      <c r="C51" s="2">
-        <v>2.0833333333333332E-2</v>
       </c>
       <c r="D51" t="s">
         <v>11</v>
@@ -2422,10 +2422,13 @@
         <v>33</v>
       </c>
       <c r="H51" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I51">
-        <v>40</v>
+        <v>39</v>
+      </c>
+      <c r="M51" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.2">
@@ -2433,25 +2436,25 @@
         <v>5</v>
       </c>
       <c r="B52" s="2">
-        <v>0.79166666666666663</v>
+        <v>1</v>
       </c>
       <c r="C52" s="2">
-        <v>0.8125</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="D52" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E52" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G52" t="s">
         <v>33</v>
       </c>
       <c r="H52" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="I52">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.2">
@@ -2459,10 +2462,10 @@
         <v>5</v>
       </c>
       <c r="B53" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C53" s="2">
         <v>0.8125</v>
-      </c>
-      <c r="C53" s="2">
-        <v>0.83333333333333304</v>
       </c>
       <c r="D53" t="s">
         <v>18</v>
@@ -2474,10 +2477,10 @@
         <v>33</v>
       </c>
       <c r="H53" t="s">
-        <v>19</v>
+        <v>96</v>
       </c>
       <c r="I53">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.2">
@@ -2485,10 +2488,10 @@
         <v>5</v>
       </c>
       <c r="B54" s="2">
+        <v>0.8125</v>
+      </c>
+      <c r="C54" s="2">
         <v>0.83333333333333304</v>
-      </c>
-      <c r="C54" s="2">
-        <v>0.875</v>
       </c>
       <c r="D54" t="s">
         <v>18</v>
@@ -2500,10 +2503,10 @@
         <v>33</v>
       </c>
       <c r="H54" t="s">
-        <v>102</v>
+        <v>19</v>
       </c>
       <c r="I54">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.2">
@@ -2511,10 +2514,10 @@
         <v>5</v>
       </c>
       <c r="B55" s="2">
+        <v>0.83333333333333304</v>
+      </c>
+      <c r="C55" s="2">
         <v>0.875</v>
-      </c>
-      <c r="C55" s="2">
-        <v>0.89583333333333404</v>
       </c>
       <c r="D55" t="s">
         <v>18</v>
@@ -2526,10 +2529,10 @@
         <v>33</v>
       </c>
       <c r="H55" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="I55">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.2">
@@ -2537,10 +2540,10 @@
         <v>5</v>
       </c>
       <c r="B56" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C56" s="2">
         <v>0.89583333333333404</v>
-      </c>
-      <c r="C56" s="2">
-        <v>0.91666666666666696</v>
       </c>
       <c r="D56" t="s">
         <v>18</v>
@@ -2552,10 +2555,10 @@
         <v>33</v>
       </c>
       <c r="H56" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="I56">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.2">
@@ -2563,10 +2566,10 @@
         <v>5</v>
       </c>
       <c r="B57" s="2">
+        <v>0.89583333333333404</v>
+      </c>
+      <c r="C57" s="2">
         <v>0.91666666666666696</v>
-      </c>
-      <c r="C57" s="2">
-        <v>0.937500000000001</v>
       </c>
       <c r="D57" t="s">
         <v>18</v>
@@ -2578,13 +2581,10 @@
         <v>33</v>
       </c>
       <c r="H57" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="I57">
-        <v>46</v>
-      </c>
-      <c r="M57" t="s">
-        <v>149</v>
+        <v>45</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.2">
@@ -2592,10 +2592,10 @@
         <v>5</v>
       </c>
       <c r="B58" s="2">
+        <v>0.91666666666666696</v>
+      </c>
+      <c r="C58" s="2">
         <v>0.937500000000001</v>
-      </c>
-      <c r="C58" s="2">
-        <v>0.95833333333333404</v>
       </c>
       <c r="D58" t="s">
         <v>18</v>
@@ -2607,13 +2607,13 @@
         <v>33</v>
       </c>
       <c r="H58" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="I58">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M58" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.2">
@@ -2621,10 +2621,10 @@
         <v>5</v>
       </c>
       <c r="B59" s="2">
+        <v>0.937500000000001</v>
+      </c>
+      <c r="C59" s="2">
         <v>0.95833333333333404</v>
-      </c>
-      <c r="C59" s="2">
-        <v>0.97916666666666696</v>
       </c>
       <c r="D59" t="s">
         <v>18</v>
@@ -2636,10 +2636,13 @@
         <v>33</v>
       </c>
       <c r="H59" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="I59">
-        <v>48</v>
+        <v>47</v>
+      </c>
+      <c r="M59" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.2">
@@ -2647,10 +2650,10 @@
         <v>5</v>
       </c>
       <c r="B60" s="2">
+        <v>0.95833333333333404</v>
+      </c>
+      <c r="C60" s="2">
         <v>0.97916666666666696</v>
-      </c>
-      <c r="C60" s="2">
-        <v>0</v>
       </c>
       <c r="D60" t="s">
         <v>18</v>
@@ -2662,10 +2665,10 @@
         <v>33</v>
       </c>
       <c r="H60" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="I60">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.2">
@@ -2673,22 +2676,25 @@
         <v>5</v>
       </c>
       <c r="B61" s="2">
-        <v>0.70833333333333337</v>
+        <v>0.97916666666666696</v>
       </c>
       <c r="C61" s="2">
-        <v>0.8125</v>
+        <v>0</v>
       </c>
       <c r="D61" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="E61" t="s">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="G61" t="s">
+        <v>33</v>
       </c>
       <c r="H61" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
       <c r="I61">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.2">
@@ -2696,10 +2702,10 @@
         <v>5</v>
       </c>
       <c r="B62" s="2">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="C62" s="2">
         <v>0.8125</v>
-      </c>
-      <c r="C62" s="2">
-        <v>0.84027777777777779</v>
       </c>
       <c r="D62" t="s">
         <v>42</v>
@@ -2707,14 +2713,11 @@
       <c r="E62" t="s">
         <v>25</v>
       </c>
-      <c r="G62" t="s">
-        <v>33</v>
-      </c>
       <c r="H62" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="I62">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.2">
@@ -2722,10 +2725,10 @@
         <v>5</v>
       </c>
       <c r="B63" s="2">
+        <v>0.8125</v>
+      </c>
+      <c r="C63" s="2">
         <v>0.84027777777777779</v>
-      </c>
-      <c r="C63" s="2">
-        <v>0.875</v>
       </c>
       <c r="D63" t="s">
         <v>42</v>
@@ -2737,10 +2740,10 @@
         <v>33</v>
       </c>
       <c r="H63" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="I63">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.2">
@@ -2748,10 +2751,10 @@
         <v>5</v>
       </c>
       <c r="B64" s="2">
+        <v>0.84027777777777779</v>
+      </c>
+      <c r="C64" s="2">
         <v>0.875</v>
-      </c>
-      <c r="C64" s="2">
-        <v>0.89583333333333337</v>
       </c>
       <c r="D64" t="s">
         <v>42</v>
@@ -2763,10 +2766,10 @@
         <v>33</v>
       </c>
       <c r="H64" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="I64">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.2">
@@ -2774,10 +2777,10 @@
         <v>5</v>
       </c>
       <c r="B65" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C65" s="2">
         <v>0.89583333333333337</v>
-      </c>
-      <c r="C65" s="2">
-        <v>0.91666666666666663</v>
       </c>
       <c r="D65" t="s">
         <v>42</v>
@@ -2789,10 +2792,10 @@
         <v>33</v>
       </c>
       <c r="H65" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="I65">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.2">
@@ -2800,10 +2803,10 @@
         <v>5</v>
       </c>
       <c r="B66" s="2">
+        <v>0.89583333333333337</v>
+      </c>
+      <c r="C66" s="2">
         <v>0.91666666666666663</v>
-      </c>
-      <c r="C66" s="2">
-        <v>0.95833333333333337</v>
       </c>
       <c r="D66" t="s">
         <v>42</v>
@@ -2815,10 +2818,10 @@
         <v>33</v>
       </c>
       <c r="H66" t="s">
-        <v>111</v>
-      </c>
-      <c r="I66" t="s">
-        <v>84</v>
+        <v>107</v>
+      </c>
+      <c r="I66">
+        <v>54</v>
       </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.2">
@@ -2826,10 +2829,10 @@
         <v>5</v>
       </c>
       <c r="B67" s="2">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="C67" s="2">
         <v>0.95833333333333337</v>
-      </c>
-      <c r="C67" s="2">
-        <v>0.97916666666666663</v>
       </c>
       <c r="D67" t="s">
         <v>42</v>
@@ -2841,10 +2844,10 @@
         <v>33</v>
       </c>
       <c r="H67" t="s">
-        <v>110</v>
-      </c>
-      <c r="I67">
-        <v>55</v>
+        <v>106</v>
+      </c>
+      <c r="I67" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.2">
@@ -2852,10 +2855,10 @@
         <v>5</v>
       </c>
       <c r="B68" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="C68" s="2">
         <v>0.97916666666666663</v>
-      </c>
-      <c r="C68" s="2">
-        <v>0</v>
       </c>
       <c r="D68" t="s">
         <v>42</v>
@@ -2867,50 +2870,47 @@
         <v>33</v>
       </c>
       <c r="H68" t="s">
+        <v>105</v>
+      </c>
+      <c r="I68">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>5</v>
+      </c>
+      <c r="B69" s="2">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="C69" s="2">
+        <v>0</v>
+      </c>
+      <c r="D69" t="s">
+        <v>42</v>
+      </c>
+      <c r="E69" t="s">
+        <v>25</v>
+      </c>
+      <c r="G69" t="s">
+        <v>33</v>
+      </c>
+      <c r="H69" t="s">
         <v>46</v>
       </c>
-      <c r="I68" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="69" spans="1:15" ht="51" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
-        <v>5</v>
-      </c>
-      <c r="B69" s="2">
+      <c r="I69" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" ht="51" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>5</v>
+      </c>
+      <c r="B70" s="2">
         <v>0.58333333333333337</v>
       </c>
-      <c r="C69" s="2">
+      <c r="C70" s="2">
         <v>0.60416666666666663</v>
-      </c>
-      <c r="D69" t="s">
-        <v>43</v>
-      </c>
-      <c r="E69" t="s">
-        <v>47</v>
-      </c>
-      <c r="F69" t="s">
-        <v>117</v>
-      </c>
-      <c r="H69" t="s">
-        <v>118</v>
-      </c>
-      <c r="I69">
-        <v>56</v>
-      </c>
-      <c r="J69" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="70" spans="1:15" ht="68" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>5</v>
-      </c>
-      <c r="B70" s="2">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="C70" s="2">
-        <v>0.625</v>
       </c>
       <c r="D70" t="s">
         <v>43</v>
@@ -2919,27 +2919,27 @@
         <v>47</v>
       </c>
       <c r="F70" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="H70" t="s">
+        <v>113</v>
+      </c>
+      <c r="I70">
+        <v>56</v>
+      </c>
+      <c r="J70" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="I70">
-        <v>57</v>
-      </c>
-      <c r="J70" s="3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="71" spans="1:15" ht="85" x14ac:dyDescent="0.2">
+    </row>
+    <row r="71" spans="1:15" ht="68" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>5</v>
       </c>
       <c r="B71" s="2">
-        <v>0.64583333333333337</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="C71" s="2">
-        <v>0.66666666666666663</v>
+        <v>0.625</v>
       </c>
       <c r="D71" t="s">
         <v>43</v>
@@ -2948,27 +2948,27 @@
         <v>47</v>
       </c>
       <c r="F71" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="H71" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="I71">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J71" s="3" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="72" spans="1:15" ht="34" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" ht="85" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>5</v>
       </c>
       <c r="B72" s="2">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="C72" s="2">
         <v>0.66666666666666663</v>
-      </c>
-      <c r="C72" s="2">
-        <v>0.6875</v>
       </c>
       <c r="D72" t="s">
         <v>43</v>
@@ -2977,112 +2977,115 @@
         <v>47</v>
       </c>
       <c r="F72" t="s">
+        <v>112</v>
+      </c>
+      <c r="H72" t="s">
+        <v>166</v>
+      </c>
+      <c r="I72">
+        <v>58</v>
+      </c>
+      <c r="J72" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="H72" t="s">
-        <v>121</v>
-      </c>
-      <c r="I72">
+    </row>
+    <row r="73" spans="1:15" ht="34" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>5</v>
+      </c>
+      <c r="B73" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C73" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="D73" t="s">
+        <v>43</v>
+      </c>
+      <c r="E73" t="s">
+        <v>47</v>
+      </c>
+      <c r="F73" t="s">
+        <v>112</v>
+      </c>
+      <c r="H73" t="s">
+        <v>115</v>
+      </c>
+      <c r="I73">
         <v>59</v>
       </c>
-      <c r="J72" s="3" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="73" spans="1:15" ht="221" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
-        <v>5</v>
-      </c>
-      <c r="B73" s="2">
+      <c r="J73" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" ht="221" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>5</v>
+      </c>
+      <c r="B74" s="2">
         <v>0.54166666666666663</v>
       </c>
-      <c r="C73" s="2">
+      <c r="C74" s="2">
         <v>0.57291666666666663</v>
       </c>
-      <c r="D73" t="s">
+      <c r="D74" t="s">
         <v>20</v>
-      </c>
-      <c r="E73" t="s">
-        <v>25</v>
-      </c>
-      <c r="F73" t="s">
-        <v>29</v>
-      </c>
-      <c r="G73" t="s">
-        <v>33</v>
-      </c>
-      <c r="H73" t="s">
-        <v>139</v>
-      </c>
-      <c r="I73">
-        <v>60</v>
-      </c>
-      <c r="J73" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="L73" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="M73" t="s">
-        <v>130</v>
-      </c>
-      <c r="N73" t="s">
-        <v>134</v>
-      </c>
-      <c r="O73" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="74" spans="1:15" ht="68" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
-        <v>5</v>
-      </c>
-      <c r="B74" s="2">
-        <v>0.9375</v>
-      </c>
-      <c r="C74" s="2">
-        <v>0</v>
-      </c>
-      <c r="D74" t="s">
-        <v>12</v>
       </c>
       <c r="E74" t="s">
         <v>25</v>
       </c>
+      <c r="F74" t="s">
+        <v>29</v>
+      </c>
+      <c r="G74" t="s">
+        <v>33</v>
+      </c>
       <c r="H74" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="I74">
+        <v>60</v>
+      </c>
+      <c r="J74" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="L74" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="M74" t="s">
+        <v>124</v>
+      </c>
+      <c r="N74" t="s">
+        <v>128</v>
+      </c>
+      <c r="O74" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" ht="68" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>5</v>
+      </c>
+      <c r="B75" s="2">
+        <v>0.9375</v>
+      </c>
+      <c r="C75" s="2">
+        <v>0</v>
+      </c>
+      <c r="D75" t="s">
+        <v>12</v>
+      </c>
+      <c r="E75" t="s">
+        <v>25</v>
+      </c>
+      <c r="H75" t="s">
+        <v>120</v>
+      </c>
+      <c r="I75">
         <v>61</v>
       </c>
-      <c r="J74" s="3" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
-        <v>5</v>
-      </c>
-      <c r="B75" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="C75" s="2">
-        <v>0.81944444444444442</v>
-      </c>
-      <c r="D75" t="s">
-        <v>43</v>
-      </c>
-      <c r="E75" t="s">
-        <v>24</v>
-      </c>
-      <c r="G75" t="s">
-        <v>33</v>
-      </c>
-      <c r="H75" t="s">
-        <v>164</v>
-      </c>
-      <c r="I75">
-        <v>62</v>
+      <c r="J75" s="3" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.2">
@@ -3090,10 +3093,10 @@
         <v>5</v>
       </c>
       <c r="B76" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C76" s="2">
         <v>0.81944444444444442</v>
-      </c>
-      <c r="C76" s="2">
-        <v>0.84722222222222221</v>
       </c>
       <c r="D76" t="s">
         <v>43</v>
@@ -3105,10 +3108,10 @@
         <v>33</v>
       </c>
       <c r="H76" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="I76">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.2">
@@ -3116,10 +3119,10 @@
         <v>5</v>
       </c>
       <c r="B77" s="2">
+        <v>0.81944444444444442</v>
+      </c>
+      <c r="C77" s="2">
         <v>0.84722222222222221</v>
-      </c>
-      <c r="C77" s="2">
-        <v>0.875</v>
       </c>
       <c r="D77" t="s">
         <v>43</v>
@@ -3131,10 +3134,10 @@
         <v>33</v>
       </c>
       <c r="H77" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="I77">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.2">
@@ -3142,10 +3145,10 @@
         <v>5</v>
       </c>
       <c r="B78" s="2">
+        <v>0.84722222222222221</v>
+      </c>
+      <c r="C78" s="2">
         <v>0.875</v>
-      </c>
-      <c r="C78" s="2">
-        <v>0.90277777777777779</v>
       </c>
       <c r="D78" t="s">
         <v>43</v>
@@ -3157,10 +3160,10 @@
         <v>33</v>
       </c>
       <c r="H78" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="I78">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.2">
@@ -3168,10 +3171,10 @@
         <v>5</v>
       </c>
       <c r="B79" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C79" s="2">
         <v>0.90277777777777779</v>
-      </c>
-      <c r="C79" s="2">
-        <v>0.93055555555555558</v>
       </c>
       <c r="D79" t="s">
         <v>43</v>
@@ -3183,10 +3186,10 @@
         <v>33</v>
       </c>
       <c r="H79" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="I79">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.2">
@@ -3194,10 +3197,10 @@
         <v>5</v>
       </c>
       <c r="B80" s="2">
+        <v>0.90277777777777779</v>
+      </c>
+      <c r="C80" s="2">
         <v>0.93055555555555558</v>
-      </c>
-      <c r="C80" s="2">
-        <v>0.95833333333333337</v>
       </c>
       <c r="D80" t="s">
         <v>43</v>
@@ -3209,10 +3212,10 @@
         <v>33</v>
       </c>
       <c r="H80" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="I80">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.2">
@@ -3220,10 +3223,10 @@
         <v>5</v>
       </c>
       <c r="B81" s="2">
+        <v>0.93055555555555558</v>
+      </c>
+      <c r="C81" s="2">
         <v>0.95833333333333337</v>
-      </c>
-      <c r="C81" s="2">
-        <v>0.98611111111111116</v>
       </c>
       <c r="D81" t="s">
         <v>43</v>
@@ -3235,10 +3238,10 @@
         <v>33</v>
       </c>
       <c r="H81" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="I81">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
@@ -3246,10 +3249,10 @@
         <v>5</v>
       </c>
       <c r="B82" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="C82" s="2">
         <v>0.98611111111111116</v>
-      </c>
-      <c r="C82" s="2">
-        <v>1.3888888888888888E-2</v>
       </c>
       <c r="D82" t="s">
         <v>43</v>
@@ -3261,9 +3264,35 @@
         <v>33</v>
       </c>
       <c r="H82" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="I82">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>5</v>
+      </c>
+      <c r="B83" s="2">
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="C83" s="2">
+        <v>1.3888888888888888E-2</v>
+      </c>
+      <c r="D83" t="s">
+        <v>43</v>
+      </c>
+      <c r="E83" t="s">
+        <v>24</v>
+      </c>
+      <c r="G83" t="s">
+        <v>33</v>
+      </c>
+      <c r="H83" t="s">
+        <v>165</v>
+      </c>
+      <c r="I83">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Removed a non-headline artist page
</commit_message>
<xml_diff>
--- a/data/lineup-2026.xlsx
+++ b/data/lineup-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pekkos/git/bingsjostamman.se/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448E422F-356C-B442-99C9-F67AE128387B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAD1C50C-9DB2-FE45-BEA8-4CDAEDF387C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="173">
   <si>
     <t>day</t>
   </si>
@@ -480,9 +480,6 @@
   </si>
   <si>
     <t>2026/storrada_ebulii.jpg</t>
-  </si>
-  <si>
-    <t>I Storrådas musik står mörkret i centrum. Det som skaver, det brustna hjärtat och den karga ensamheten. Men längst in i mörkret finns också ljuset. Glädjen, kärleken och samhörigheten. Med rykande fiolspel, drivande gitarr och kraftfull sång, ofta i stämmor, utforskar Storråda mörkrets alla vrår och skrymslen, med en stark grund i den nordiska folkmusiktraditionen.  Storråda består av Alma Strang Brydevall, Pella Wig &amp; Olle Westling</t>
   </si>
   <si>
     <t>https://www.tabyspelmansgille.se/</t>
@@ -1333,13 +1330,13 @@
         <v>5</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>41</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -1539,7 +1536,7 @@
         <v>0.5</v>
       </c>
       <c r="D19" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E19" t="s">
         <v>47</v>
@@ -1566,7 +1563,7 @@
         <v>0.47916666666666669</v>
       </c>
       <c r="D20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E20" t="s">
         <v>47</v>
@@ -1578,7 +1575,7 @@
         <v>12</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K20" s="1"/>
     </row>
@@ -1605,7 +1602,7 @@
         <v>13</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1625,13 +1622,13 @@
         <v>47</v>
       </c>
       <c r="H22" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I22">
         <v>135</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="102" x14ac:dyDescent="0.2">
@@ -1735,7 +1732,7 @@
         <v>17</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1767,7 +1764,7 @@
         <v>34</v>
       </c>
       <c r="K27" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1828,10 +1825,10 @@
         <v>66</v>
       </c>
       <c r="K29" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="M29" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1863,7 +1860,7 @@
         <v>65</v>
       </c>
       <c r="K30" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1944,7 +1941,7 @@
         <v>24</v>
       </c>
       <c r="K33" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
@@ -2051,10 +2048,10 @@
         <v>27</v>
       </c>
       <c r="K37" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="M37" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
@@ -2083,7 +2080,7 @@
         <v>32</v>
       </c>
       <c r="K38" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
@@ -2112,7 +2109,7 @@
         <v>28</v>
       </c>
       <c r="M39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
@@ -2375,9 +2372,7 @@
       <c r="I49">
         <v>37</v>
       </c>
-      <c r="L49" s="7" t="s">
-        <v>148</v>
-      </c>
+      <c r="L49" s="7"/>
       <c r="M49" t="s">
         <v>147</v>
       </c>
@@ -2986,7 +2981,7 @@
         <v>112</v>
       </c>
       <c r="H72" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I72">
         <v>58</v>
@@ -3114,7 +3109,7 @@
         <v>33</v>
       </c>
       <c r="H76" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I76">
         <v>62</v>
@@ -3140,7 +3135,7 @@
         <v>33</v>
       </c>
       <c r="H77" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I77">
         <v>63</v>
@@ -3166,7 +3161,7 @@
         <v>33</v>
       </c>
       <c r="H78" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I78">
         <v>64</v>
@@ -3192,7 +3187,7 @@
         <v>33</v>
       </c>
       <c r="H79" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I79">
         <v>65</v>
@@ -3218,7 +3213,7 @@
         <v>33</v>
       </c>
       <c r="H80" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I80">
         <v>66</v>
@@ -3244,7 +3239,7 @@
         <v>33</v>
       </c>
       <c r="H81" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I81">
         <v>67</v>
@@ -3270,7 +3265,7 @@
         <v>33</v>
       </c>
       <c r="H82" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I82">
         <v>68</v>
@@ -3296,7 +3291,7 @@
         <v>33</v>
       </c>
       <c r="H83" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I83">
         <v>69</v>

</xml_diff>

<commit_message>
Lineup updates and corrections
</commit_message>
<xml_diff>
--- a/data/lineup-2026.xlsx
+++ b/data/lineup-2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pekkos/git/bingsjostamman.se/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAD1C50C-9DB2-FE45-BEA8-4CDAEDF387C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5AA48AE-38AD-CD46-B2E6-E6B8C5BC79F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="178">
   <si>
     <t>day</t>
   </si>
@@ -146,9 +146,6 @@
     <t>Östen med resten</t>
   </si>
   <si>
-    <t>Systrar med bröder</t>
-  </si>
-  <si>
     <t>Besserbotten Band</t>
   </si>
   <si>
@@ -416,9 +413,6 @@
     <t>2026/merit-hemmingson_jws0da.jpg</t>
   </si>
   <si>
-    <t>2026/polenta_pcjvf6.jpg</t>
-  </si>
-  <si>
     <t>eyebrow</t>
   </si>
   <si>
@@ -434,9 +428,6 @@
     <t>Under årets spelmansmöte ska "stråken få tala". Uttrycket anspelar på bevingade ord från en av spelmanssveriges giganter, Hjort Anders Olsson, som hade sitt hem i Bingsjö - tvärs över vägen från Nygårdsgården. Vi får stifta bekantskap med denna portalfigur för Bingsjömusiken genom toner och ord förmedlade av Anders Bjernulf, Ola Bäckström, Jonas Päckos, Täpp Jenny Nylander, Johan Nylander och Anders Junkas. Efter konserten visas en utställning med fokus på Hjort Anders och andra bingsjöspelmän i det vita "posthuset" tvärd över gården från konsertlokalen. Entré löses på plats på Nygårdsgården. Swish eller kontant.</t>
   </si>
   <si>
-    <t>Söderut är det mat, österut är det ett slangord för "stamp" men på den finska folkmusikhimlen är Polenta ett åttaarmat musikaliskt vidunder. Ett tätt samspel och öppenhet för influenser utmärker Polentas halsbrytande och svindlande musikanteri och de blandar sin musik med lika delar tradition, förnyelse och spelglädje. Polenta spelar förutom under invigningsprogrammet på Dansbanan också på Bystuguscenen under tisdagkvällen.</t>
-  </si>
-  <si>
     <t>Hjort Anders i ord och toner</t>
   </si>
   <si>
@@ -464,18 +455,12 @@
     <t>Spelmannen Hjort Anders Olsson hyllas med konsert och ny utställning. I toner och ord får vi stifta bekantskap med denna legendariska fiolspelman.</t>
   </si>
   <si>
-    <t>För många år sedan besökte orgelspelmannen Merit Hemmingson Bingsjöstämman. Musiken, luften och slänten upp mot Päkkosgården satte ett avtryck och sådde ett frö. Nu återvänder Merit med en fullmogen skiva, fylld med Pekkos Pers musik i elektrisk skrud. Tillsammans med trummis och slagverkare fyller hon Bingsjö kapell med välbekanta Bingsjölåtar på sitt eget sätt. Skivsläppet äger rum ett stenkast från gården där Pekkos Per levde under 1800-talet. Gården är kvar i släkten och här tog Päkkos Gustaf emot spel- och fikasugna Bingsjöstämmobesökare i över tre decennier. Pekkos Per &amp; jag presenteras under invigningsprogrammet på Dansbanan innan kvällens konserter i kapellet.</t>
-  </si>
-  <si>
     <t>2026/peter-jeanett_ectmjb.jpg</t>
   </si>
   <si>
     <t>2026/folke-amy_bfh8dg.jpg</t>
   </si>
   <si>
-    <t>2026/alvina-herbinger-rygne_sebdup.jpg</t>
-  </si>
-  <si>
     <t>2026/vatmark_rndjfm.jpg</t>
   </si>
   <si>
@@ -555,6 +540,36 @@
   </si>
   <si>
     <t>Från spelmansstämmor och lastbilsflak till radio- och tv-program och vidare till final i Melodifestivalen i Globen. Och nu landar Östen med resten i Bingsjö. En återkomst till spelmansstämmor, alltså, medan bandets 40-åriga historia bara fortsätter.</t>
+  </si>
+  <si>
+    <t>I Storrådas musik står mörkret i centrum. Det som skaver, det brustna hjärtat och den karga ensamheten. Men längst in i mörkret finns också ljuset. Glädjen, kärleken och samhörigheten. Med rykande fiolspel, drivande gitarr och kraftfull sång, ofta i stämmor, utforskar Storråda mörkrets alla vrår och skrymslen, med en stark grund i den nordiska folkmusiktraditionen.  Storråda består av Alma Strang Brydevall, Pella Wig &amp; Olle Westling.</t>
+  </si>
+  <si>
+    <t>https://vadurmusic.com/</t>
+  </si>
+  <si>
+    <t>Med rötter i den nordiska folkmusiken komponerar VÄDUR eget material influerat av medlemmarnas olika musikaliska bakgrund. Resultatet blir en blandning av stämningsfulla stråkmelodier, varvat med rytmiskt fokus och ett groove som får rummet att gunga. Fyra starka personliga uttryck och musikaliska bakgrunder flätas sömlöst samman på scenen till en gemensam kraft som lockar med sig både inbitna folkmusiker och nyfikna vardagslyssnare. Vädur är Evelina Eriksson, Maria ten Wolde, Kentaro Ragert &amp; Jakob Rolandsson</t>
+  </si>
+  <si>
+    <t>2026/vadur_jcpysl.jpg</t>
+  </si>
+  <si>
+    <t>2026/polenta2_piz5a6.jpg</t>
+  </si>
+  <si>
+    <t>Det är sällsynt att stöta på ett band så samspelt som Polenta. Denna finska åttahänta organism andas, rör sig och dansar som en enda enhet, där tre fioler och en gitarr samverkar i perfekt harmoni. Den samlade energin från de fyra musikerna flödar som en elektrisk ström och förmedlar både djupet i den nordiska traditionen, pulsen i den moderna folkmusiken och den rena glädjen i att skapa musik tillsammans. I fotspåren av giganter som JPP, Frigg och Väsen hämtar Polenta kraft ur de djupa och livfulla rötterna i den nordiska fiolmusiken. Här väntar virtuosa melodier, finurligt vävda stämmor och dynamiska, organiska rytmer som tillsammans skapar ett sound som känns både tidlöst och djärvt. Polenta är en favorit på den finska folkdansscenen, och deras drivande rytmer lockar publiken till rörelse – vare sig det handlar om att stampa takten med foten, gunga med i musiken eller helt ge sig hän åt dansgolvet. Polenta är Aino Kinnunen, Veera Kuisma, Olli Sippola &amp; Mikko Malmivaara.</t>
+  </si>
+  <si>
+    <t>Pekkos Per har för mej alltid varit en av dom absolut tyngsta namnen inom svensk folkmusik, berättar Merit Hemmingson. ”Många av hans låtar går i både dur och moll, vilket för mej är både klurigt och spännande. Låtarna har mestadels spelats av fiolspelmän, men här vill jag förmedla dom på ett annat och otraditionellt sätt på mitt favoritinstrument Hammond B3.” Merit Hemmingson har ägnat livet åt att utforska och konstruera sitt egna musikaliska landskap. De både böjer och utmanar genres på sätt som ofta skapat svallvågor i omgivningen. Hennes personliga uttryck har sedan 60-talet skapat ett unikt utrymme i svensk musikhistoria där jazz, grooverock och framför allt folkmusik möts. Under våren har Merit spelat in delar av Pekkos Pers låtskatt i en nytolkning som är lika bekant och tydlig som virvlande, inspirerad och utforskande. Nu ger Merit sig ut på turné tillsammans med sitt band. Vad kan passa bättre än att börja resan i Bingsjö kapell under Bingsjöstämman, inom synhåll från gården där Pekkos Per levde under 1800-talet?</t>
+  </si>
+  <si>
+    <t>Systrar &amp; bröder</t>
+  </si>
+  <si>
+    <t>2026/alvina-kvartett_rief24.jpg</t>
+  </si>
+  <si>
+    <t>2026/ville-tommie_lgvnkq.jpg</t>
   </si>
 </sst>
 </file>
@@ -564,7 +579,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="h:mm;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -599,6 +614,12 @@
       <name val="Helvetica Neue"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -621,7 +642,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -633,7 +654,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="20" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -969,7 +998,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F23F1BC-D35E-3E42-8F88-5D61ED802479}">
-  <dimension ref="A1:O83"/>
+  <dimension ref="A1:O84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.83203125" bestFit="1" customWidth="1"/>
@@ -981,7 +1010,7 @@
     <col min="9" max="9" width="10.33203125" customWidth="1"/>
     <col min="10" max="10" width="48.5" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="32" customWidth="1"/>
-    <col min="12" max="12" width="43.6640625" style="3" customWidth="1"/>
+    <col min="12" max="12" width="43.6640625" style="7" customWidth="1"/>
     <col min="13" max="13" width="33.5" customWidth="1"/>
     <col min="14" max="14" width="28.5" customWidth="1"/>
     <col min="15" max="15" width="35.6640625" customWidth="1"/>
@@ -1021,20 +1050,20 @@
       <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="7" t="s">
         <v>27</v>
       </c>
       <c r="M1" t="s">
         <v>3</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="O1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" ht="238" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="372" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1057,28 +1086,28 @@
         <v>33</v>
       </c>
       <c r="H2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J2" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="K2" t="s">
+        <v>122</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="M2" t="s">
+        <v>124</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="O2" t="s">
         <v>136</v>
-      </c>
-      <c r="K2" t="s">
-        <v>123</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="M2" t="s">
-        <v>125</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="O2" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
@@ -1101,13 +1130,13 @@
         <v>33</v>
       </c>
       <c r="H3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="51" x14ac:dyDescent="0.2">
@@ -1124,10 +1153,10 @@
         <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I4">
         <v>1</v>
@@ -1147,10 +1176,10 @@
         <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I5">
         <v>2</v>
@@ -1170,7 +1199,7 @@
         <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G6" t="s">
         <v>33</v>
@@ -1179,7 +1208,7 @@
         <v>17</v>
       </c>
       <c r="I6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="34" x14ac:dyDescent="0.2">
@@ -1196,10 +1225,10 @@
         <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I7">
         <v>3</v>
@@ -1219,22 +1248,22 @@
         <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G8" t="s">
         <v>33</v>
       </c>
       <c r="H8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="153" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="340" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1248,7 +1277,7 @@
         <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F9" t="s">
         <v>29</v>
@@ -1257,28 +1286,28 @@
         <v>33</v>
       </c>
       <c r="H9" t="s">
+        <v>38</v>
+      </c>
+      <c r="I9" t="s">
+        <v>79</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="K9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="I9" t="s">
-        <v>80</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>132</v>
+      <c r="L9" s="7" t="s">
+        <v>173</v>
       </c>
       <c r="M9" t="s">
-        <v>126</v>
+        <v>172</v>
       </c>
       <c r="N9" t="s">
+        <v>134</v>
+      </c>
+      <c r="O9" t="s">
         <v>137</v>
-      </c>
-      <c r="O9" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="17" x14ac:dyDescent="0.2">
@@ -1295,10 +1324,10 @@
         <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I10">
         <v>4</v>
@@ -1330,13 +1359,13 @@
         <v>5</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -1350,7 +1379,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E12" t="s">
         <v>25</v>
@@ -1359,7 +1388,7 @@
         <v>33</v>
       </c>
       <c r="H12" t="s">
-        <v>36</v>
+        <v>175</v>
       </c>
       <c r="I12">
         <v>6</v>
@@ -1377,7 +1406,7 @@
         <v>0.83333333333333304</v>
       </c>
       <c r="D13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E13" t="s">
         <v>25</v>
@@ -1386,14 +1415,14 @@
         <v>33</v>
       </c>
       <c r="H13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I13">
         <v>7</v>
       </c>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" ht="166" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1404,7 +1433,7 @@
         <v>0.875</v>
       </c>
       <c r="D14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E14" t="s">
         <v>25</v>
@@ -1413,12 +1442,20 @@
         <v>33</v>
       </c>
       <c r="H14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I14">
         <v>8</v>
       </c>
-      <c r="K14" s="1"/>
+      <c r="K14" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="L14" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="M14" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -1431,7 +1468,7 @@
         <v>0.91666666666666696</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E15" t="s">
         <v>25</v>
@@ -1440,10 +1477,10 @@
         <v>33</v>
       </c>
       <c r="H15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
@@ -1457,7 +1494,7 @@
         <v>0.95833333333333304</v>
       </c>
       <c r="D16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E16" t="s">
         <v>25</v>
@@ -1466,7 +1503,7 @@
         <v>33</v>
       </c>
       <c r="H16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I16">
         <v>9</v>
@@ -1478,22 +1515,25 @@
         <v>4</v>
       </c>
       <c r="B17" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="C17" s="2">
         <v>0.79166666666666663</v>
       </c>
-      <c r="C17" s="2">
-        <v>0.875</v>
-      </c>
       <c r="D17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E17" t="s">
         <v>24</v>
       </c>
+      <c r="G17" t="s">
+        <v>33</v>
+      </c>
       <c r="H17" t="s">
-        <v>45</v>
-      </c>
-      <c r="I17">
         <v>10</v>
+      </c>
+      <c r="I17" t="s">
+        <v>32</v>
       </c>
       <c r="K17" s="1"/>
     </row>
@@ -1502,110 +1542,108 @@
         <v>4</v>
       </c>
       <c r="B18" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C18" s="2">
         <v>0.875</v>
       </c>
-      <c r="C18" s="2">
-        <v>0.91666666666666663</v>
-      </c>
       <c r="D18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E18" t="s">
         <v>24</v>
       </c>
-      <c r="G18" t="s">
-        <v>33</v>
-      </c>
       <c r="H18" t="s">
+        <v>44</v>
+      </c>
+      <c r="I18">
+        <v>10</v>
+      </c>
+      <c r="K18" s="1"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C19" s="2">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="D19" t="s">
+        <v>42</v>
+      </c>
+      <c r="E19" t="s">
+        <v>24</v>
+      </c>
+      <c r="G19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H19" t="s">
+        <v>45</v>
+      </c>
+      <c r="I19" t="s">
+        <v>103</v>
+      </c>
+      <c r="J19" s="4"/>
+      <c r="K19" s="1"/>
+    </row>
+    <row r="20" spans="1:13" ht="68" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="2">
+        <v>0.375</v>
+      </c>
+      <c r="C20" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D20" t="s">
+        <v>162</v>
+      </c>
+      <c r="E20" t="s">
         <v>46</v>
       </c>
-      <c r="I18" t="s">
-        <v>104</v>
-      </c>
-      <c r="J18" s="4"/>
-      <c r="K18" s="1"/>
-    </row>
-    <row r="19" spans="1:13" ht="68" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" s="2">
-        <v>0.375</v>
-      </c>
-      <c r="C19" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="D19" t="s">
-        <v>167</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="H20" t="s">
         <v>47</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I20">
+        <v>11</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="K20" s="1"/>
+    </row>
+    <row r="21" spans="1:13" ht="85" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="2">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="C21" s="2">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="D21" t="s">
+        <v>162</v>
+      </c>
+      <c r="E21" t="s">
+        <v>46</v>
+      </c>
+      <c r="H21" t="s">
         <v>48</v>
       </c>
-      <c r="I19">
-        <v>11</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="K19" s="1"/>
-    </row>
-    <row r="20" spans="1:13" ht="85" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" s="2">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="C20" s="2">
-        <v>0.47916666666666669</v>
-      </c>
-      <c r="D20" t="s">
-        <v>167</v>
-      </c>
-      <c r="E20" t="s">
-        <v>47</v>
-      </c>
-      <c r="H20" t="s">
-        <v>49</v>
-      </c>
-      <c r="I20">
+      <c r="I21">
         <v>12</v>
       </c>
-      <c r="J20" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="K20" s="1"/>
-    </row>
-    <row r="21" spans="1:13" ht="51" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" s="2">
-        <v>0.625</v>
-      </c>
-      <c r="C21" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-      <c r="D21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E21" t="s">
-        <v>47</v>
-      </c>
-      <c r="H21" t="s">
-        <v>14</v>
-      </c>
-      <c r="I21">
-        <v>13</v>
-      </c>
       <c r="J21" s="3" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+        <v>161</v>
+      </c>
+      <c r="K21" s="1"/>
+    </row>
+    <row r="22" spans="1:13" ht="51" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>5</v>
       </c>
@@ -1613,158 +1651,152 @@
         <v>0.625</v>
       </c>
       <c r="C22" s="2">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D22" t="s">
+        <v>50</v>
+      </c>
+      <c r="E22" t="s">
+        <v>46</v>
+      </c>
+      <c r="H22" t="s">
+        <v>14</v>
+      </c>
+      <c r="I22">
+        <v>13</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="C23" s="2">
         <v>0.79166666666666663</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D23" t="s">
+        <v>50</v>
+      </c>
+      <c r="E23" t="s">
+        <v>46</v>
+      </c>
+      <c r="H23" t="s">
+        <v>164</v>
+      </c>
+      <c r="I23">
+        <v>135</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="102" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="2">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C24" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="D24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" t="s">
+        <v>46</v>
+      </c>
+      <c r="H24" t="s">
         <v>51</v>
       </c>
-      <c r="E22" t="s">
-        <v>47</v>
-      </c>
-      <c r="H22" t="s">
-        <v>169</v>
-      </c>
-      <c r="I22">
-        <v>135</v>
-      </c>
-      <c r="J22" s="3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" ht="102" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" s="2">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="C23" s="2">
-        <v>0.75</v>
-      </c>
-      <c r="D23" t="s">
-        <v>13</v>
-      </c>
-      <c r="E23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H23" t="s">
+      <c r="I24">
+        <v>14</v>
+      </c>
+      <c r="J24" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I23">
-        <v>14</v>
-      </c>
-      <c r="J23" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="68" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" s="2">
+    </row>
+    <row r="25" spans="1:13" ht="68" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" s="2">
         <v>0.45833333333333331</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C25" s="2">
         <v>0.54166666666666663</v>
-      </c>
-      <c r="D24" t="s">
-        <v>18</v>
-      </c>
-      <c r="E24" t="s">
-        <v>54</v>
-      </c>
-      <c r="H24" t="s">
-        <v>55</v>
-      </c>
-      <c r="I24">
-        <v>15</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" ht="51" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>5</v>
-      </c>
-      <c r="B25" s="2">
-        <v>0.64583333333333337</v>
-      </c>
-      <c r="C25" s="2">
-        <v>0.6875</v>
       </c>
       <c r="D25" t="s">
         <v>18</v>
       </c>
       <c r="E25" t="s">
+        <v>53</v>
+      </c>
+      <c r="H25" t="s">
         <v>54</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25">
+        <v>15</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="51" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" s="2">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="C26" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="D26" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26" t="s">
+        <v>53</v>
+      </c>
+      <c r="H26" t="s">
+        <v>56</v>
+      </c>
+      <c r="I26">
+        <v>16</v>
+      </c>
+      <c r="J26" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="I25">
-        <v>16</v>
-      </c>
-      <c r="J25" s="3" t="s">
+    </row>
+    <row r="27" spans="1:13" ht="68" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" s="2">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="C27" s="2">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="D27" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" ht="68" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>5</v>
-      </c>
-      <c r="B26" s="2">
-        <v>0.85416666666666663</v>
-      </c>
-      <c r="C26" s="2">
-        <v>0.91666666666666663</v>
-      </c>
-      <c r="D26" t="s">
-        <v>59</v>
-      </c>
-      <c r="E26" t="s">
+      <c r="E27" t="s">
         <v>26</v>
       </c>
-      <c r="H26" t="s">
+      <c r="H27" t="s">
         <v>15</v>
       </c>
-      <c r="I26">
+      <c r="I27">
         <v>17</v>
       </c>
-      <c r="J26" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" ht="17" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>5</v>
-      </c>
-      <c r="B27" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="C27" s="2">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="D27" t="s">
-        <v>16</v>
-      </c>
-      <c r="E27" t="s">
-        <v>23</v>
-      </c>
-      <c r="G27" t="s">
-        <v>33</v>
-      </c>
-      <c r="H27" t="s">
-        <v>10</v>
-      </c>
-      <c r="I27" t="s">
-        <v>32</v>
-      </c>
       <c r="J27" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="K27" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1772,10 +1804,10 @@
         <v>5</v>
       </c>
       <c r="B28" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C28" s="2">
         <v>0.83333333333333337</v>
-      </c>
-      <c r="C28" s="2">
-        <v>0.875</v>
       </c>
       <c r="D28" t="s">
         <v>16</v>
@@ -1787,13 +1819,16 @@
         <v>33</v>
       </c>
       <c r="H28" t="s">
-        <v>60</v>
-      </c>
-      <c r="I28">
-        <v>19</v>
+        <v>10</v>
+      </c>
+      <c r="I28" t="s">
+        <v>32</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>67</v>
+        <v>34</v>
+      </c>
+      <c r="K28" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1801,10 +1836,10 @@
         <v>5</v>
       </c>
       <c r="B29" s="2">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="C29" s="2">
         <v>0.875</v>
-      </c>
-      <c r="C29" s="2">
-        <v>0.91666666666666696</v>
       </c>
       <c r="D29" t="s">
         <v>16</v>
@@ -1816,30 +1851,24 @@
         <v>33</v>
       </c>
       <c r="H29" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I29">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J29" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="K29" t="s">
-        <v>150</v>
-      </c>
-      <c r="M29" t="s">
-        <v>152</v>
-      </c>
     </row>
     <row r="30" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>5</v>
       </c>
       <c r="B30" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C30" s="2">
         <v>0.91666666666666696</v>
-      </c>
-      <c r="C30" s="2">
-        <v>0.95833333333333304</v>
       </c>
       <c r="D30" t="s">
         <v>16</v>
@@ -1851,16 +1880,19 @@
         <v>33</v>
       </c>
       <c r="H30" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I30">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J30" s="3" t="s">
         <v>65</v>
       </c>
       <c r="K30" t="s">
-        <v>155</v>
+        <v>145</v>
+      </c>
+      <c r="M30" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="17" x14ac:dyDescent="0.2">
@@ -1868,10 +1900,10 @@
         <v>5</v>
       </c>
       <c r="B31" s="2">
-        <v>0.95833333333333404</v>
+        <v>0.91666666666666696</v>
       </c>
       <c r="C31" s="2">
-        <v>1</v>
+        <v>0.95833333333333304</v>
       </c>
       <c r="D31" t="s">
         <v>16</v>
@@ -1883,36 +1915,45 @@
         <v>33</v>
       </c>
       <c r="H31" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I31">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J31" s="3" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K31" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>5</v>
       </c>
       <c r="B32" s="2">
-        <v>0.625</v>
+        <v>0.95833333333333404</v>
       </c>
       <c r="C32" s="2">
-        <v>0.79166666666666663</v>
+        <v>1</v>
       </c>
       <c r="D32" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E32" t="s">
-        <v>25</v>
+        <v>23</v>
+      </c>
+      <c r="G32" t="s">
+        <v>33</v>
       </c>
       <c r="H32" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I32">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
@@ -1920,39 +1961,33 @@
         <v>5</v>
       </c>
       <c r="B33" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="C33" s="2">
         <v>0.79166666666666663</v>
-      </c>
-      <c r="C33" s="2">
-        <v>0.83333333333333337</v>
       </c>
       <c r="D33" t="s">
         <v>21</v>
       </c>
       <c r="E33" t="s">
-        <v>24</v>
-      </c>
-      <c r="G33" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="H33" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I33">
-        <v>24</v>
-      </c>
-      <c r="K33" t="s">
-        <v>151</v>
+        <v>23</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>5</v>
       </c>
-      <c r="B34" s="6">
+      <c r="B34" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C34" s="2">
         <v>0.83333333333333337</v>
-      </c>
-      <c r="C34" s="2">
-        <v>0.86111111111111116</v>
       </c>
       <c r="D34" t="s">
         <v>21</v>
@@ -1964,21 +1999,24 @@
         <v>33</v>
       </c>
       <c r="H34" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="I34">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="K34" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>5</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35" s="6">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="C35" s="2">
         <v>0.86111111111111116</v>
-      </c>
-      <c r="C35" s="2">
-        <v>0.90277777777777779</v>
       </c>
       <c r="D35" t="s">
         <v>21</v>
@@ -1992,8 +2030,8 @@
       <c r="H35" t="s">
         <v>77</v>
       </c>
-      <c r="I35" t="s">
-        <v>79</v>
+      <c r="I35">
+        <v>25</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
@@ -2001,10 +2039,10 @@
         <v>5</v>
       </c>
       <c r="B36" s="2">
+        <v>0.86111111111111116</v>
+      </c>
+      <c r="C36" s="2">
         <v>0.90277777777777779</v>
-      </c>
-      <c r="C36" s="2">
-        <v>0.93055555555555558</v>
       </c>
       <c r="D36" t="s">
         <v>21</v>
@@ -2018,8 +2056,8 @@
       <c r="H36" t="s">
         <v>76</v>
       </c>
-      <c r="I36">
-        <v>26</v>
+      <c r="I36" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
@@ -2027,10 +2065,10 @@
         <v>5</v>
       </c>
       <c r="B37" s="2">
+        <v>0.90277777777777779</v>
+      </c>
+      <c r="C37" s="2">
         <v>0.93055555555555558</v>
-      </c>
-      <c r="C37" s="2">
-        <v>0.95833333333333337</v>
       </c>
       <c r="D37" t="s">
         <v>21</v>
@@ -2045,13 +2083,7 @@
         <v>75</v>
       </c>
       <c r="I37">
-        <v>27</v>
-      </c>
-      <c r="K37" t="s">
-        <v>149</v>
-      </c>
-      <c r="M37" t="s">
-        <v>153</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
@@ -2059,10 +2091,10 @@
         <v>5</v>
       </c>
       <c r="B38" s="2">
+        <v>0.93055555555555558</v>
+      </c>
+      <c r="C38" s="2">
         <v>0.95833333333333337</v>
-      </c>
-      <c r="C38" s="2">
-        <v>0.98611111111111116</v>
       </c>
       <c r="D38" t="s">
         <v>21</v>
@@ -2076,10 +2108,13 @@
       <c r="H38" t="s">
         <v>74</v>
       </c>
-      <c r="I38" t="s">
-        <v>32</v>
+      <c r="I38">
+        <v>27</v>
       </c>
       <c r="K38" t="s">
+        <v>144</v>
+      </c>
+      <c r="M38" t="s">
         <v>148</v>
       </c>
     </row>
@@ -2088,10 +2123,10 @@
         <v>5</v>
       </c>
       <c r="B39" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="C39" s="2">
         <v>0.98611111111111116</v>
-      </c>
-      <c r="C39" s="2">
-        <v>1.3888888888888888E-2</v>
       </c>
       <c r="D39" t="s">
         <v>21</v>
@@ -2105,11 +2140,11 @@
       <c r="H39" t="s">
         <v>73</v>
       </c>
-      <c r="I39">
-        <v>28</v>
-      </c>
-      <c r="M39" t="s">
-        <v>154</v>
+      <c r="I39" t="s">
+        <v>32</v>
+      </c>
+      <c r="K39" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
@@ -2117,10 +2152,10 @@
         <v>5</v>
       </c>
       <c r="B40" s="2">
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="C40" s="2">
         <v>1.3888888888888888E-2</v>
-      </c>
-      <c r="C40" s="2">
-        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D40" t="s">
         <v>21</v>
@@ -2135,7 +2170,10 @@
         <v>72</v>
       </c>
       <c r="I40">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="M40" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
@@ -2143,10 +2181,10 @@
         <v>5</v>
       </c>
       <c r="B41" s="2">
+        <v>1.3888888888888888E-2</v>
+      </c>
+      <c r="C41" s="2">
         <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C41" s="2">
-        <v>6.9444444444444448E-2</v>
       </c>
       <c r="D41" t="s">
         <v>21</v>
@@ -2161,7 +2199,7 @@
         <v>71</v>
       </c>
       <c r="I41">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
@@ -2169,28 +2207,25 @@
         <v>5</v>
       </c>
       <c r="B42" s="2">
-        <v>0.79166666666666663</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="C42" s="2">
-        <v>0.8125</v>
+        <v>6.9444444444444448E-2</v>
       </c>
       <c r="D42" t="s">
         <v>21</v>
       </c>
       <c r="E42" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G42" t="s">
         <v>33</v>
       </c>
       <c r="H42" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="I42">
-        <v>31</v>
-      </c>
-      <c r="M42" t="s">
-        <v>145</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
@@ -2198,10 +2233,10 @@
         <v>5</v>
       </c>
       <c r="B43" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C43" s="2">
         <v>0.8125</v>
-      </c>
-      <c r="C43" s="2">
-        <v>0.83333333333333304</v>
       </c>
       <c r="D43" t="s">
         <v>11</v>
@@ -2213,22 +2248,24 @@
         <v>33</v>
       </c>
       <c r="H43" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I43">
-        <v>32</v>
-      </c>
-      <c r="K43" s="1"/>
+        <v>31</v>
+      </c>
+      <c r="M43" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>5</v>
       </c>
       <c r="B44" s="2">
+        <v>0.8125</v>
+      </c>
+      <c r="C44" s="2">
         <v>0.83333333333333304</v>
-      </c>
-      <c r="C44" s="2">
-        <v>0.85416666666666696</v>
       </c>
       <c r="D44" t="s">
         <v>11</v>
@@ -2240,21 +2277,22 @@
         <v>33</v>
       </c>
       <c r="H44" t="s">
-        <v>17</v>
-      </c>
-      <c r="I44" t="s">
-        <v>79</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="I44">
+        <v>32</v>
+      </c>
+      <c r="K44" s="1"/>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>5</v>
       </c>
       <c r="B45" s="2">
+        <v>0.83333333333333304</v>
+      </c>
+      <c r="C45" s="2">
         <v>0.85416666666666696</v>
-      </c>
-      <c r="C45" s="2">
-        <v>0.875</v>
       </c>
       <c r="D45" t="s">
         <v>11</v>
@@ -2262,11 +2300,14 @@
       <c r="E45" t="s">
         <v>25</v>
       </c>
+      <c r="G45" t="s">
+        <v>33</v>
+      </c>
       <c r="H45" t="s">
-        <v>89</v>
-      </c>
-      <c r="I45">
-        <v>33</v>
+        <v>17</v>
+      </c>
+      <c r="I45" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
@@ -2274,10 +2315,10 @@
         <v>5</v>
       </c>
       <c r="B46" s="2">
+        <v>0.85416666666666696</v>
+      </c>
+      <c r="C46" s="2">
         <v>0.875</v>
-      </c>
-      <c r="C46" s="2">
-        <v>0.89583333333333404</v>
       </c>
       <c r="D46" t="s">
         <v>11</v>
@@ -2285,14 +2326,11 @@
       <c r="E46" t="s">
         <v>25</v>
       </c>
-      <c r="G46" t="s">
-        <v>33</v>
-      </c>
       <c r="H46" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I46">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
@@ -2300,10 +2338,10 @@
         <v>5</v>
       </c>
       <c r="B47" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C47" s="2">
         <v>0.89583333333333404</v>
-      </c>
-      <c r="C47" s="2">
-        <v>0.91666666666666696</v>
       </c>
       <c r="D47" t="s">
         <v>11</v>
@@ -2315,10 +2353,10 @@
         <v>33</v>
       </c>
       <c r="H47" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="I47">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.2">
@@ -2326,10 +2364,10 @@
         <v>5</v>
       </c>
       <c r="B48" s="2">
+        <v>0.89583333333333404</v>
+      </c>
+      <c r="C48" s="2">
         <v>0.91666666666666696</v>
-      </c>
-      <c r="C48" s="2">
-        <v>0.937500000000001</v>
       </c>
       <c r="D48" t="s">
         <v>11</v>
@@ -2341,21 +2379,21 @@
         <v>33</v>
       </c>
       <c r="H48" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="I48">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>5</v>
       </c>
       <c r="B49" s="2">
+        <v>0.91666666666666696</v>
+      </c>
+      <c r="C49" s="2">
         <v>0.937500000000001</v>
-      </c>
-      <c r="C49" s="2">
-        <v>0.95833333333333404</v>
       </c>
       <c r="D49" t="s">
         <v>11</v>
@@ -2367,25 +2405,21 @@
         <v>33</v>
       </c>
       <c r="H49" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="I49">
-        <v>37</v>
-      </c>
-      <c r="L49" s="7"/>
-      <c r="M49" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" ht="216" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>5</v>
       </c>
       <c r="B50" s="2">
+        <v>0.937500000000001</v>
+      </c>
+      <c r="C50" s="2">
         <v>0.95833333333333404</v>
-      </c>
-      <c r="C50" s="2">
-        <v>0.97916666666666696</v>
       </c>
       <c r="D50" t="s">
         <v>11</v>
@@ -2397,10 +2431,16 @@
         <v>33</v>
       </c>
       <c r="H50" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="I50">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="L50" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="M50" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.2">
@@ -2408,10 +2448,10 @@
         <v>5</v>
       </c>
       <c r="B51" s="2">
+        <v>0.95833333333333404</v>
+      </c>
+      <c r="C51" s="2">
         <v>0.97916666666666696</v>
-      </c>
-      <c r="C51" s="2">
-        <v>1</v>
       </c>
       <c r="D51" t="s">
         <v>11</v>
@@ -2423,13 +2463,10 @@
         <v>33</v>
       </c>
       <c r="H51" t="s">
-        <v>94</v>
+        <v>121</v>
       </c>
       <c r="I51">
-        <v>39</v>
-      </c>
-      <c r="M51" t="s">
-        <v>146</v>
+        <v>38</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.2">
@@ -2437,10 +2474,10 @@
         <v>5</v>
       </c>
       <c r="B52" s="2">
+        <v>0.97916666666666696</v>
+      </c>
+      <c r="C52" s="2">
         <v>1</v>
-      </c>
-      <c r="C52" s="2">
-        <v>2.0833333333333332E-2</v>
       </c>
       <c r="D52" t="s">
         <v>11</v>
@@ -2452,10 +2489,13 @@
         <v>33</v>
       </c>
       <c r="H52" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="I52">
-        <v>40</v>
+        <v>39</v>
+      </c>
+      <c r="M52" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.2">
@@ -2463,25 +2503,25 @@
         <v>5</v>
       </c>
       <c r="B53" s="2">
-        <v>0.79166666666666663</v>
+        <v>1</v>
       </c>
       <c r="C53" s="2">
-        <v>0.8125</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="D53" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E53" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G53" t="s">
         <v>33</v>
       </c>
       <c r="H53" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I53">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.2">
@@ -2489,10 +2529,10 @@
         <v>5</v>
       </c>
       <c r="B54" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C54" s="2">
         <v>0.8125</v>
-      </c>
-      <c r="C54" s="2">
-        <v>0.83333333333333304</v>
       </c>
       <c r="D54" t="s">
         <v>18</v>
@@ -2504,10 +2544,10 @@
         <v>33</v>
       </c>
       <c r="H54" t="s">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="I54">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.2">
@@ -2515,10 +2555,10 @@
         <v>5</v>
       </c>
       <c r="B55" s="2">
+        <v>0.8125</v>
+      </c>
+      <c r="C55" s="2">
         <v>0.83333333333333304</v>
-      </c>
-      <c r="C55" s="2">
-        <v>0.875</v>
       </c>
       <c r="D55" t="s">
         <v>18</v>
@@ -2530,10 +2570,10 @@
         <v>33</v>
       </c>
       <c r="H55" t="s">
-        <v>97</v>
+        <v>19</v>
       </c>
       <c r="I55">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.2">
@@ -2541,10 +2581,10 @@
         <v>5</v>
       </c>
       <c r="B56" s="2">
+        <v>0.83333333333333304</v>
+      </c>
+      <c r="C56" s="2">
         <v>0.875</v>
-      </c>
-      <c r="C56" s="2">
-        <v>0.89583333333333404</v>
       </c>
       <c r="D56" t="s">
         <v>18</v>
@@ -2556,10 +2596,10 @@
         <v>33</v>
       </c>
       <c r="H56" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I56">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.2">
@@ -2567,10 +2607,10 @@
         <v>5</v>
       </c>
       <c r="B57" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C57" s="2">
         <v>0.89583333333333404</v>
-      </c>
-      <c r="C57" s="2">
-        <v>0.91666666666666696</v>
       </c>
       <c r="D57" t="s">
         <v>18</v>
@@ -2582,10 +2622,13 @@
         <v>33</v>
       </c>
       <c r="H57" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="I57">
-        <v>45</v>
+        <v>44</v>
+      </c>
+      <c r="M57" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.2">
@@ -2593,10 +2636,10 @@
         <v>5</v>
       </c>
       <c r="B58" s="2">
+        <v>0.89583333333333404</v>
+      </c>
+      <c r="C58" s="2">
         <v>0.91666666666666696</v>
-      </c>
-      <c r="C58" s="2">
-        <v>0.937500000000001</v>
       </c>
       <c r="D58" t="s">
         <v>18</v>
@@ -2608,13 +2651,10 @@
         <v>33</v>
       </c>
       <c r="H58" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I58">
-        <v>46</v>
-      </c>
-      <c r="M58" t="s">
-        <v>143</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.2">
@@ -2622,10 +2662,10 @@
         <v>5</v>
       </c>
       <c r="B59" s="2">
+        <v>0.91666666666666696</v>
+      </c>
+      <c r="C59" s="2">
         <v>0.937500000000001</v>
-      </c>
-      <c r="C59" s="2">
-        <v>0.95833333333333404</v>
       </c>
       <c r="D59" t="s">
         <v>18</v>
@@ -2637,13 +2677,13 @@
         <v>33</v>
       </c>
       <c r="H59" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I59">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M59" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.2">
@@ -2651,10 +2691,10 @@
         <v>5</v>
       </c>
       <c r="B60" s="2">
+        <v>0.937500000000001</v>
+      </c>
+      <c r="C60" s="2">
         <v>0.95833333333333404</v>
-      </c>
-      <c r="C60" s="2">
-        <v>0.97916666666666696</v>
       </c>
       <c r="D60" t="s">
         <v>18</v>
@@ -2666,10 +2706,13 @@
         <v>33</v>
       </c>
       <c r="H60" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I60">
-        <v>48</v>
+        <v>47</v>
+      </c>
+      <c r="M60" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.2">
@@ -2677,10 +2720,10 @@
         <v>5</v>
       </c>
       <c r="B61" s="2">
+        <v>0.95833333333333404</v>
+      </c>
+      <c r="C61" s="2">
         <v>0.97916666666666696</v>
-      </c>
-      <c r="C61" s="2">
-        <v>0</v>
       </c>
       <c r="D61" t="s">
         <v>18</v>
@@ -2692,10 +2735,10 @@
         <v>33</v>
       </c>
       <c r="H61" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I61">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.2">
@@ -2703,22 +2746,25 @@
         <v>5</v>
       </c>
       <c r="B62" s="2">
-        <v>0.70833333333333337</v>
+        <v>0.97916666666666696</v>
       </c>
       <c r="C62" s="2">
-        <v>0.8125</v>
+        <v>0</v>
       </c>
       <c r="D62" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="E62" t="s">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="G62" t="s">
+        <v>33</v>
       </c>
       <c r="H62" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="I62">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.2">
@@ -2726,25 +2772,22 @@
         <v>5</v>
       </c>
       <c r="B63" s="2">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="C63" s="2">
         <v>0.8125</v>
       </c>
-      <c r="C63" s="2">
-        <v>0.84027777777777779</v>
-      </c>
       <c r="D63" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E63" t="s">
         <v>25</v>
       </c>
-      <c r="G63" t="s">
-        <v>33</v>
-      </c>
       <c r="H63" t="s">
         <v>110</v>
       </c>
       <c r="I63">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.2">
@@ -2752,13 +2795,13 @@
         <v>5</v>
       </c>
       <c r="B64" s="2">
+        <v>0.8125</v>
+      </c>
+      <c r="C64" s="2">
         <v>0.84027777777777779</v>
       </c>
-      <c r="C64" s="2">
-        <v>0.875</v>
-      </c>
       <c r="D64" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E64" t="s">
         <v>25</v>
@@ -2770,7 +2813,7 @@
         <v>109</v>
       </c>
       <c r="I64">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.2">
@@ -2778,13 +2821,13 @@
         <v>5</v>
       </c>
       <c r="B65" s="2">
+        <v>0.84027777777777779</v>
+      </c>
+      <c r="C65" s="2">
         <v>0.875</v>
       </c>
-      <c r="C65" s="2">
-        <v>0.89583333333333337</v>
-      </c>
       <c r="D65" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E65" t="s">
         <v>25</v>
@@ -2796,7 +2839,7 @@
         <v>108</v>
       </c>
       <c r="I65">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.2">
@@ -2804,13 +2847,13 @@
         <v>5</v>
       </c>
       <c r="B66" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C66" s="2">
         <v>0.89583333333333337</v>
       </c>
-      <c r="C66" s="2">
-        <v>0.91666666666666663</v>
-      </c>
       <c r="D66" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E66" t="s">
         <v>25</v>
@@ -2822,7 +2865,7 @@
         <v>107</v>
       </c>
       <c r="I66">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.2">
@@ -2830,13 +2873,13 @@
         <v>5</v>
       </c>
       <c r="B67" s="2">
+        <v>0.89583333333333337</v>
+      </c>
+      <c r="C67" s="2">
         <v>0.91666666666666663</v>
       </c>
-      <c r="C67" s="2">
-        <v>0.95833333333333337</v>
-      </c>
       <c r="D67" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E67" t="s">
         <v>25</v>
@@ -2847,8 +2890,8 @@
       <c r="H67" t="s">
         <v>106</v>
       </c>
-      <c r="I67" t="s">
-        <v>79</v>
+      <c r="I67">
+        <v>54</v>
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.2">
@@ -2856,13 +2899,13 @@
         <v>5</v>
       </c>
       <c r="B68" s="2">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="C68" s="2">
         <v>0.95833333333333337</v>
       </c>
-      <c r="C68" s="2">
-        <v>0.97916666666666663</v>
-      </c>
       <c r="D68" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E68" t="s">
         <v>25</v>
@@ -2873,8 +2916,8 @@
       <c r="H68" t="s">
         <v>105</v>
       </c>
-      <c r="I68">
-        <v>55</v>
+      <c r="I68" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.2">
@@ -2882,13 +2925,13 @@
         <v>5</v>
       </c>
       <c r="B69" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="C69" s="2">
         <v>0.97916666666666663</v>
       </c>
-      <c r="C69" s="2">
-        <v>0</v>
-      </c>
       <c r="D69" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E69" t="s">
         <v>25</v>
@@ -2897,222 +2940,222 @@
         <v>33</v>
       </c>
       <c r="H69" t="s">
+        <v>104</v>
+      </c>
+      <c r="I69">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>5</v>
+      </c>
+      <c r="B70" s="2">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="C70" s="2">
+        <v>0</v>
+      </c>
+      <c r="D70" t="s">
+        <v>41</v>
+      </c>
+      <c r="E70" t="s">
+        <v>25</v>
+      </c>
+      <c r="G70" t="s">
+        <v>33</v>
+      </c>
+      <c r="H70" t="s">
+        <v>45</v>
+      </c>
+      <c r="I70" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" ht="51" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>5</v>
+      </c>
+      <c r="B71" s="2">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C71" s="2">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D71" t="s">
+        <v>42</v>
+      </c>
+      <c r="E71" t="s">
         <v>46</v>
       </c>
-      <c r="I69" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="70" spans="1:15" ht="51" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>5</v>
-      </c>
-      <c r="B70" s="2">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="C70" s="2">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="D70" t="s">
-        <v>43</v>
-      </c>
-      <c r="E70" t="s">
-        <v>47</v>
-      </c>
-      <c r="F70" t="s">
+      <c r="F71" t="s">
+        <v>111</v>
+      </c>
+      <c r="H71" t="s">
         <v>112</v>
       </c>
-      <c r="H70" t="s">
-        <v>113</v>
-      </c>
-      <c r="I70">
+      <c r="I71">
         <v>56</v>
-      </c>
-      <c r="J70" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="71" spans="1:15" ht="68" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
-        <v>5</v>
-      </c>
-      <c r="B71" s="2">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="C71" s="2">
-        <v>0.625</v>
-      </c>
-      <c r="D71" t="s">
-        <v>43</v>
-      </c>
-      <c r="E71" t="s">
-        <v>47</v>
-      </c>
-      <c r="F71" t="s">
-        <v>112</v>
-      </c>
-      <c r="H71" t="s">
-        <v>114</v>
-      </c>
-      <c r="I71">
-        <v>57</v>
       </c>
       <c r="J71" s="3" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="72" spans="1:15" ht="85" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:15" ht="68" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>5</v>
       </c>
       <c r="B72" s="2">
-        <v>0.64583333333333337</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="C72" s="2">
-        <v>0.66666666666666663</v>
+        <v>0.625</v>
       </c>
       <c r="D72" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E72" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F72" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H72" t="s">
-        <v>165</v>
+        <v>113</v>
       </c>
       <c r="I72">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J72" s="3" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="73" spans="1:15" ht="34" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:15" ht="85" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>5</v>
       </c>
       <c r="B73" s="2">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="C73" s="2">
         <v>0.66666666666666663</v>
       </c>
-      <c r="C73" s="2">
-        <v>0.6875</v>
-      </c>
       <c r="D73" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E73" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F73" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H73" t="s">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="I73">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J73" s="3" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="74" spans="1:15" ht="221" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:15" ht="34" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>5</v>
       </c>
       <c r="B74" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C74" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="D74" t="s">
+        <v>42</v>
+      </c>
+      <c r="E74" t="s">
+        <v>46</v>
+      </c>
+      <c r="F74" t="s">
+        <v>111</v>
+      </c>
+      <c r="H74" t="s">
+        <v>114</v>
+      </c>
+      <c r="I74">
+        <v>59</v>
+      </c>
+      <c r="J74" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" ht="221" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>5</v>
+      </c>
+      <c r="B75" s="2">
         <v>0.54166666666666663</v>
       </c>
-      <c r="C74" s="2">
+      <c r="C75" s="2">
         <v>0.57291666666666663</v>
       </c>
-      <c r="D74" t="s">
+      <c r="D75" t="s">
         <v>20</v>
-      </c>
-      <c r="E74" t="s">
-        <v>25</v>
-      </c>
-      <c r="F74" t="s">
-        <v>29</v>
-      </c>
-      <c r="G74" t="s">
-        <v>33</v>
-      </c>
-      <c r="H74" t="s">
-        <v>133</v>
-      </c>
-      <c r="I74">
-        <v>60</v>
-      </c>
-      <c r="J74" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="L74" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="M74" t="s">
-        <v>124</v>
-      </c>
-      <c r="N74" t="s">
-        <v>128</v>
-      </c>
-      <c r="O74" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="75" spans="1:15" ht="68" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
-        <v>5</v>
-      </c>
-      <c r="B75" s="2">
-        <v>0.9375</v>
-      </c>
-      <c r="C75" s="2">
-        <v>0</v>
-      </c>
-      <c r="D75" t="s">
-        <v>12</v>
       </c>
       <c r="E75" t="s">
         <v>25</v>
       </c>
+      <c r="F75" t="s">
+        <v>29</v>
+      </c>
+      <c r="G75" t="s">
+        <v>33</v>
+      </c>
       <c r="H75" t="s">
+        <v>130</v>
+      </c>
+      <c r="I75">
+        <v>60</v>
+      </c>
+      <c r="J75" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="L75" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="M75" t="s">
+        <v>123</v>
+      </c>
+      <c r="N75" t="s">
+        <v>126</v>
+      </c>
+      <c r="O75" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" ht="68" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>5</v>
+      </c>
+      <c r="B76" s="2">
+        <v>0.9375</v>
+      </c>
+      <c r="C76" s="2">
+        <v>0</v>
+      </c>
+      <c r="D76" t="s">
+        <v>12</v>
+      </c>
+      <c r="E76" t="s">
+        <v>25</v>
+      </c>
+      <c r="H76" t="s">
+        <v>119</v>
+      </c>
+      <c r="I76">
+        <v>61</v>
+      </c>
+      <c r="J76" s="3" t="s">
         <v>120</v>
-      </c>
-      <c r="I75">
-        <v>61</v>
-      </c>
-      <c r="J75" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
-        <v>5</v>
-      </c>
-      <c r="B76" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="C76" s="2">
-        <v>0.81944444444444442</v>
-      </c>
-      <c r="D76" t="s">
-        <v>43</v>
-      </c>
-      <c r="E76" t="s">
-        <v>24</v>
-      </c>
-      <c r="G76" t="s">
-        <v>33</v>
-      </c>
-      <c r="H76" t="s">
-        <v>157</v>
-      </c>
-      <c r="I76">
-        <v>62</v>
       </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.2">
@@ -3120,13 +3163,13 @@
         <v>5</v>
       </c>
       <c r="B77" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C77" s="2">
         <v>0.81944444444444442</v>
       </c>
-      <c r="C77" s="2">
-        <v>0.84722222222222221</v>
-      </c>
       <c r="D77" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E77" t="s">
         <v>24</v>
@@ -3135,10 +3178,10 @@
         <v>33</v>
       </c>
       <c r="H77" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="I77">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.2">
@@ -3146,13 +3189,13 @@
         <v>5</v>
       </c>
       <c r="B78" s="2">
+        <v>0.81944444444444442</v>
+      </c>
+      <c r="C78" s="2">
         <v>0.84722222222222221</v>
       </c>
-      <c r="C78" s="2">
-        <v>0.875</v>
-      </c>
       <c r="D78" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E78" t="s">
         <v>24</v>
@@ -3161,10 +3204,10 @@
         <v>33</v>
       </c>
       <c r="H78" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="I78">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.2">
@@ -3172,13 +3215,13 @@
         <v>5</v>
       </c>
       <c r="B79" s="2">
+        <v>0.84722222222222221</v>
+      </c>
+      <c r="C79" s="2">
         <v>0.875</v>
       </c>
-      <c r="C79" s="2">
-        <v>0.90277777777777779</v>
-      </c>
       <c r="D79" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E79" t="s">
         <v>24</v>
@@ -3187,10 +3230,10 @@
         <v>33</v>
       </c>
       <c r="H79" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="I79">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.2">
@@ -3198,13 +3241,13 @@
         <v>5</v>
       </c>
       <c r="B80" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="C80" s="2">
         <v>0.90277777777777779</v>
       </c>
-      <c r="C80" s="2">
-        <v>0.93055555555555558</v>
-      </c>
       <c r="D80" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E80" t="s">
         <v>24</v>
@@ -3213,10 +3256,10 @@
         <v>33</v>
       </c>
       <c r="H80" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="I80">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.2">
@@ -3224,13 +3267,13 @@
         <v>5</v>
       </c>
       <c r="B81" s="2">
+        <v>0.90277777777777779</v>
+      </c>
+      <c r="C81" s="2">
         <v>0.93055555555555558</v>
       </c>
-      <c r="C81" s="2">
-        <v>0.95833333333333337</v>
-      </c>
       <c r="D81" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E81" t="s">
         <v>24</v>
@@ -3239,10 +3282,10 @@
         <v>33</v>
       </c>
       <c r="H81" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="I81">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
@@ -3250,13 +3293,13 @@
         <v>5</v>
       </c>
       <c r="B82" s="2">
+        <v>0.93055555555555558</v>
+      </c>
+      <c r="C82" s="2">
         <v>0.95833333333333337</v>
       </c>
-      <c r="C82" s="2">
-        <v>0.98611111111111116</v>
-      </c>
       <c r="D82" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E82" t="s">
         <v>24</v>
@@ -3265,10 +3308,10 @@
         <v>33</v>
       </c>
       <c r="H82" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="I82">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.2">
@@ -3276,13 +3319,13 @@
         <v>5</v>
       </c>
       <c r="B83" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="C83" s="2">
         <v>0.98611111111111116</v>
       </c>
-      <c r="C83" s="2">
-        <v>1.3888888888888888E-2</v>
-      </c>
       <c r="D83" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E83" t="s">
         <v>24</v>
@@ -3291,13 +3334,42 @@
         <v>33</v>
       </c>
       <c r="H83" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="I83">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>5</v>
+      </c>
+      <c r="B84" s="2">
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="C84" s="2">
+        <v>1.3888888888888888E-2</v>
+      </c>
+      <c r="D84" t="s">
+        <v>42</v>
+      </c>
+      <c r="E84" t="s">
+        <v>24</v>
+      </c>
+      <c r="G84" t="s">
+        <v>33</v>
+      </c>
+      <c r="H84" t="s">
+        <v>159</v>
+      </c>
+      <c r="I84">
         <v>69</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="K14" r:id="rId1" xr:uid="{8ED0E742-6A4A-844E-8645-5EC84E48241E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Act name changed, redirected artist page
</commit_message>
<xml_diff>
--- a/data/lineup-2026.xlsx
+++ b/data/lineup-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pekkos/git/bingsjostamman.se/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02303AA5-3CF7-B145-9F6D-495AB0F81C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BFF60F8-83B6-3143-8CFD-6049B0A1B69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="44600" windowHeight="31460" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -149,9 +149,6 @@
     <t>Besserbotten Band</t>
   </si>
   <si>
-    <t>Vädur</t>
-  </si>
-  <si>
     <t>Polenta</t>
   </si>
   <si>
@@ -569,12 +566,6 @@
     <t>Fyra starka personliga uttryck och musikaliska bakgrunder flätas sömlöst samman på scenen till en gemensam kraft som lockar med sig både inbitna folkmusiker och nyfikna vardagslyssnare.</t>
   </si>
   <si>
-    <t xml:space="preserve">Med rötter i den nordiska folkmusiken komponerar VÄDUR eget material influerat av medlemmarnas olika musikaliska bakgrund. Resultatet blir en blandning av stämningsfulla stråkmelodier, varvat med rytmiskt fokus och ett groove som får rummet att gunga.  </t>
-  </si>
-  <si>
-    <t>Vädur är Evelina Eriksson, Maria ten Wolde, Kentaro Ragert &amp; Jakob Rolandsson</t>
-  </si>
-  <si>
     <t>Elsa &amp; Alma</t>
   </si>
   <si>
@@ -615,6 +606,15 @@
   </si>
   <si>
     <t>2026/alma-elsa_yn1kqs.jpg</t>
+  </si>
+  <si>
+    <t>Vaedur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Med rötter i den nordiska folkmusiken komponerar VAEDUR eget material influerat av medlemmarnas olika musikaliska bakgrund. Resultatet blir en blandning av stämningsfulla stråkmelodier, varvat med rytmiskt fokus och ett groove som får rummet att gunga.  </t>
+  </si>
+  <si>
+    <t>Vaedur är Evelina Eriksson, Maria ten Wolde, Kentaro Ragert &amp; Jakob Rolandsson</t>
   </si>
 </sst>
 </file>
@@ -1145,19 +1145,19 @@
         <v>27</v>
       </c>
       <c r="M1" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="N1" s="5" t="s">
         <v>171</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>172</v>
       </c>
       <c r="O1" s="6" t="s">
         <v>3</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="136" x14ac:dyDescent="0.2">
@@ -1183,34 +1183,34 @@
         <v>33</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="O2" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
@@ -1233,13 +1233,13 @@
         <v>33</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="51" x14ac:dyDescent="0.2">
@@ -1256,10 +1256,10 @@
         <v>21</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I4" s="8">
         <v>1</v>
@@ -1279,10 +1279,10 @@
         <v>21</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I5" s="8">
         <v>2</v>
@@ -1302,7 +1302,7 @@
         <v>21</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>33</v>
@@ -1311,7 +1311,7 @@
         <v>17</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="34" x14ac:dyDescent="0.2">
@@ -1328,10 +1328,10 @@
         <v>21</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I7" s="8">
         <v>3</v>
@@ -1351,19 +1351,19 @@
         <v>21</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>33</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="170" x14ac:dyDescent="0.2">
@@ -1380,7 +1380,7 @@
         <v>21</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>29</v>
@@ -1389,34 +1389,34 @@
         <v>33</v>
       </c>
       <c r="H9" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>39</v>
-      </c>
       <c r="L9" s="3" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="O9" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P9" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="17" x14ac:dyDescent="0.2">
@@ -1433,10 +1433,10 @@
         <v>21</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I10" s="8">
         <v>4</v>
@@ -1468,13 +1468,13 @@
         <v>5</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
@@ -1488,7 +1488,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>25</v>
@@ -1497,7 +1497,7 @@
         <v>33</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I12" s="8">
         <v>6</v>
@@ -1515,7 +1515,7 @@
         <v>0.83333333333333304</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>25</v>
@@ -1542,7 +1542,7 @@
         <v>0.875</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>25</v>
@@ -1551,28 +1551,28 @@
         <v>33</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>37</v>
+        <v>190</v>
       </c>
       <c r="I14" s="8">
         <v>8</v>
       </c>
       <c r="K14" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="N14" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="O14" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="L14" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="M14" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="N14" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="O14" s="8" t="s">
-        <v>163</v>
-      </c>
       <c r="Q14" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
@@ -1586,7 +1586,7 @@
         <v>0.91666666666666696</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>25</v>
@@ -1595,10 +1595,10 @@
         <v>33</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
@@ -1612,7 +1612,7 @@
         <v>0.95833333333333304</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>25</v>
@@ -1621,7 +1621,7 @@
         <v>33</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I16" s="8">
         <v>9</v>
@@ -1639,7 +1639,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>24</v>
@@ -1666,13 +1666,13 @@
         <v>0.875</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>24</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I18" s="8">
         <v>10</v>
@@ -1690,7 +1690,7 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>24</v>
@@ -1699,10 +1699,10 @@
         <v>33</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J19" s="12"/>
       <c r="K19" s="10"/>
@@ -1718,19 +1718,19 @@
         <v>0.5</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E20" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="H20" s="8" t="s">
         <v>46</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>47</v>
       </c>
       <c r="I20" s="8">
         <v>11</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K20" s="10"/>
     </row>
@@ -1745,19 +1745,19 @@
         <v>0.47916666666666669</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I21" s="8">
         <v>12</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K21" s="10"/>
     </row>
@@ -1772,10 +1772,10 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H22" s="8" t="s">
         <v>14</v>
@@ -1784,7 +1784,7 @@
         <v>13</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
@@ -1798,13 +1798,13 @@
         <v>0.6875</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I23" s="8">
         <v>99</v>
@@ -1824,16 +1824,16 @@
         <v>13</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I24" s="8">
         <v>14</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:15" ht="68" x14ac:dyDescent="0.2">
@@ -1850,16 +1850,16 @@
         <v>18</v>
       </c>
       <c r="E25" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H25" s="8" t="s">
         <v>53</v>
-      </c>
-      <c r="H25" s="8" t="s">
-        <v>54</v>
       </c>
       <c r="I25" s="8">
         <v>15</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" spans="1:15" ht="51" x14ac:dyDescent="0.2">
@@ -1876,16 +1876,16 @@
         <v>18</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I26" s="8">
         <v>16</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" spans="1:15" ht="68" x14ac:dyDescent="0.2">
@@ -1899,7 +1899,7 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E27" s="8" t="s">
         <v>26</v>
@@ -1911,7 +1911,7 @@
         <v>17</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:15" ht="17" x14ac:dyDescent="0.2">
@@ -1943,7 +1943,7 @@
         <v>34</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="29" spans="1:15" ht="17" x14ac:dyDescent="0.2">
@@ -1966,13 +1966,13 @@
         <v>33</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I29" s="8">
         <v>19</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30" spans="1:15" ht="17" x14ac:dyDescent="0.2">
@@ -1995,19 +1995,19 @@
         <v>33</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I30" s="8">
         <v>20</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O30" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="31" spans="1:15" ht="17" x14ac:dyDescent="0.2">
@@ -2030,16 +2030,16 @@
         <v>33</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I31" s="8">
         <v>21</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K31" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="32" spans="1:15" ht="17" x14ac:dyDescent="0.2">
@@ -2062,13 +2062,13 @@
         <v>33</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I32" s="8">
         <v>22</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
@@ -2088,7 +2088,7 @@
         <v>25</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I33" s="8">
         <v>23</v>
@@ -2114,13 +2114,13 @@
         <v>33</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I34" s="8">
         <v>24</v>
       </c>
       <c r="K34" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.2">
@@ -2143,7 +2143,7 @@
         <v>33</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I35" s="8">
         <v>25</v>
@@ -2169,10 +2169,10 @@
         <v>33</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.2">
@@ -2195,7 +2195,7 @@
         <v>33</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I37" s="8">
         <v>26</v>
@@ -2221,16 +2221,16 @@
         <v>33</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I38" s="8">
         <v>27</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O38" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.2">
@@ -2253,13 +2253,13 @@
         <v>33</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>32</v>
       </c>
       <c r="K39" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.2">
@@ -2282,13 +2282,13 @@
         <v>33</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I40" s="8">
         <v>28</v>
       </c>
       <c r="O40" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.2">
@@ -2311,7 +2311,7 @@
         <v>33</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I41" s="8">
         <v>29</v>
@@ -2337,7 +2337,7 @@
         <v>33</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I42" s="8">
         <v>30</v>
@@ -2363,13 +2363,13 @@
         <v>33</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I43" s="8">
         <v>31</v>
       </c>
       <c r="O43" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.2">
@@ -2392,7 +2392,7 @@
         <v>33</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I44" s="8">
         <v>32</v>
@@ -2422,7 +2422,7 @@
         <v>17</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.2">
@@ -2442,7 +2442,7 @@
         <v>25</v>
       </c>
       <c r="H46" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I46" s="8">
         <v>33</v>
@@ -2468,7 +2468,7 @@
         <v>33</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I47" s="8">
         <v>34</v>
@@ -2494,7 +2494,7 @@
         <v>33</v>
       </c>
       <c r="H48" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I48" s="8">
         <v>35</v>
@@ -2520,7 +2520,7 @@
         <v>33</v>
       </c>
       <c r="H49" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I49" s="8">
         <v>36</v>
@@ -2546,25 +2546,25 @@
         <v>33</v>
       </c>
       <c r="H50" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I50" s="8">
         <v>37</v>
       </c>
       <c r="L50" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="M50" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N50" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="M50" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="N50" s="14" t="s">
-        <v>175</v>
-      </c>
       <c r="O50" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Q50" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.2">
@@ -2587,7 +2587,7 @@
         <v>33</v>
       </c>
       <c r="H51" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I51" s="8">
         <v>38</v>
@@ -2613,13 +2613,13 @@
         <v>33</v>
       </c>
       <c r="H52" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I52" s="8">
         <v>39</v>
       </c>
       <c r="O52" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.2">
@@ -2642,7 +2642,7 @@
         <v>33</v>
       </c>
       <c r="H53" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I53" s="8">
         <v>40</v>
@@ -2668,7 +2668,7 @@
         <v>33</v>
       </c>
       <c r="H54" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I54" s="8">
         <v>41</v>
@@ -2720,7 +2720,7 @@
         <v>33</v>
       </c>
       <c r="H56" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I56" s="8">
         <v>43</v>
@@ -2746,13 +2746,13 @@
         <v>33</v>
       </c>
       <c r="H57" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I57" s="8">
         <v>44</v>
       </c>
       <c r="O57" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.2">
@@ -2775,7 +2775,7 @@
         <v>33</v>
       </c>
       <c r="H58" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I58" s="8">
         <v>45</v>
@@ -2801,13 +2801,13 @@
         <v>33</v>
       </c>
       <c r="H59" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I59" s="8">
         <v>46</v>
       </c>
       <c r="O59" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.2">
@@ -2830,13 +2830,13 @@
         <v>33</v>
       </c>
       <c r="H60" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I60" s="8">
         <v>47</v>
       </c>
       <c r="O60" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.2">
@@ -2859,7 +2859,7 @@
         <v>33</v>
       </c>
       <c r="H61" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I61" s="8">
         <v>48</v>
@@ -2885,7 +2885,7 @@
         <v>33</v>
       </c>
       <c r="H62" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I62" s="8">
         <v>49</v>
@@ -2902,13 +2902,13 @@
         <v>0.8125</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E63" s="8" t="s">
         <v>25</v>
       </c>
       <c r="H63" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I63" s="8">
         <v>50</v>
@@ -2925,7 +2925,7 @@
         <v>0.84027777777777779</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E64" s="8" t="s">
         <v>25</v>
@@ -2934,7 +2934,7 @@
         <v>33</v>
       </c>
       <c r="H64" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I64" s="8">
         <v>51</v>
@@ -2951,7 +2951,7 @@
         <v>0.875</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E65" s="8" t="s">
         <v>25</v>
@@ -2960,7 +2960,7 @@
         <v>33</v>
       </c>
       <c r="H65" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I65" s="8">
         <v>52</v>
@@ -2977,7 +2977,7 @@
         <v>0.89583333333333337</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E66" s="8" t="s">
         <v>25</v>
@@ -2986,22 +2986,22 @@
         <v>33</v>
       </c>
       <c r="H66" s="8" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="I66" s="8">
         <v>53</v>
       </c>
       <c r="L66" s="15" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="M66" s="3" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="O66" s="8" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="Q66" s="1" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.2">
@@ -3015,7 +3015,7 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E67" s="8" t="s">
         <v>25</v>
@@ -3024,7 +3024,7 @@
         <v>33</v>
       </c>
       <c r="H67" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I67" s="8">
         <v>54</v>
@@ -3041,7 +3041,7 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E68" s="8" t="s">
         <v>25</v>
@@ -3050,10 +3050,10 @@
         <v>33</v>
       </c>
       <c r="H68" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I68" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.2">
@@ -3067,7 +3067,7 @@
         <v>0.97916666666666663</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E69" s="8" t="s">
         <v>25</v>
@@ -3076,7 +3076,7 @@
         <v>33</v>
       </c>
       <c r="H69" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I69" s="8">
         <v>55</v>
@@ -3093,7 +3093,7 @@
         <v>0</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E70" s="8" t="s">
         <v>25</v>
@@ -3102,10 +3102,10 @@
         <v>33</v>
       </c>
       <c r="H70" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I70" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="71" spans="1:17" ht="51" x14ac:dyDescent="0.2">
@@ -3119,22 +3119,22 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E71" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="F71" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="H71" s="8" t="s">
         <v>109</v>
-      </c>
-      <c r="F71" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="H71" s="8" t="s">
-        <v>110</v>
       </c>
       <c r="I71" s="8">
         <v>56</v>
       </c>
       <c r="J71" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="72" spans="1:17" ht="68" x14ac:dyDescent="0.2">
@@ -3148,22 +3148,22 @@
         <v>0.625</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F72" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H72" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I72" s="8">
         <v>57</v>
       </c>
       <c r="J72" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="73" spans="1:17" ht="85" x14ac:dyDescent="0.2">
@@ -3177,22 +3177,22 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H73" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I73" s="8">
         <v>58</v>
       </c>
       <c r="J73" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="74" spans="1:17" ht="34" x14ac:dyDescent="0.2">
@@ -3206,22 +3206,22 @@
         <v>0.6875</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E74" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F74" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H74" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I74" s="8">
         <v>59</v>
       </c>
       <c r="J74" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="75" spans="1:17" ht="85" x14ac:dyDescent="0.2">
@@ -3247,31 +3247,31 @@
         <v>33</v>
       </c>
       <c r="H75" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I75" s="8">
         <v>60</v>
       </c>
       <c r="J75" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="L75" s="3" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="M75" s="3" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="N75" s="3" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="O75" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="P75" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="Q75" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="76" spans="1:17" ht="68" x14ac:dyDescent="0.2">
@@ -3291,13 +3291,13 @@
         <v>25</v>
       </c>
       <c r="H76" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I76" s="8">
         <v>61</v>
       </c>
       <c r="J76" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.2">
@@ -3311,7 +3311,7 @@
         <v>0.81944444444444442</v>
       </c>
       <c r="D77" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E77" s="8" t="s">
         <v>24</v>
@@ -3320,7 +3320,7 @@
         <v>33</v>
       </c>
       <c r="H77" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I77" s="8">
         <v>62</v>
@@ -3337,7 +3337,7 @@
         <v>0.84722222222222221</v>
       </c>
       <c r="D78" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E78" s="8" t="s">
         <v>24</v>
@@ -3346,7 +3346,7 @@
         <v>33</v>
       </c>
       <c r="H78" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I78" s="8">
         <v>63</v>
@@ -3363,7 +3363,7 @@
         <v>0.875</v>
       </c>
       <c r="D79" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E79" s="8" t="s">
         <v>24</v>
@@ -3372,7 +3372,7 @@
         <v>33</v>
       </c>
       <c r="H79" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I79" s="8">
         <v>64</v>
@@ -3389,7 +3389,7 @@
         <v>0.90277777777777779</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E80" s="8" t="s">
         <v>24</v>
@@ -3398,7 +3398,7 @@
         <v>33</v>
       </c>
       <c r="H80" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I80" s="8">
         <v>65</v>
@@ -3415,7 +3415,7 @@
         <v>0.93055555555555558</v>
       </c>
       <c r="D81" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E81" s="8" t="s">
         <v>24</v>
@@ -3424,7 +3424,7 @@
         <v>33</v>
       </c>
       <c r="H81" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I81" s="8">
         <v>66</v>
@@ -3441,7 +3441,7 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="D82" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E82" s="8" t="s">
         <v>24</v>
@@ -3450,7 +3450,7 @@
         <v>33</v>
       </c>
       <c r="H82" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I82" s="8">
         <v>67</v>
@@ -3467,7 +3467,7 @@
         <v>0.98611111111111116</v>
       </c>
       <c r="D83" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E83" s="8" t="s">
         <v>24</v>
@@ -3476,7 +3476,7 @@
         <v>33</v>
       </c>
       <c r="H83" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I83" s="8">
         <v>68</v>
@@ -3493,7 +3493,7 @@
         <v>1.3888888888888888E-2</v>
       </c>
       <c r="D84" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E84" s="8" t="s">
         <v>24</v>
@@ -3502,7 +3502,7 @@
         <v>33</v>
       </c>
       <c r="H84" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I84" s="8">
         <v>69</v>

</xml_diff>

<commit_message>
New slot and tunes update
</commit_message>
<xml_diff>
--- a/data/lineup-2026.xlsx
+++ b/data/lineup-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pekkos/git/bingsjostamman.se/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA76B9C-7D3A-0E49-B8DB-918EBBE2F9D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE6B8A4F-A735-7144-8462-43B040F7B871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="195">
   <si>
     <t>day</t>
   </si>
@@ -615,6 +615,12 @@
   </si>
   <si>
     <t>Välkomna till Barnens Bingsjö! Vi öppnar programmet med ett alldeles eget allspel för små och stora. Låtarna hittar du på sidan Allspel.</t>
+  </si>
+  <si>
+    <t>Lär dig en låt</t>
+  </si>
+  <si>
+    <t>Träffa musikanterna i bandet Vaedur och lär dig spela Fusk Olles schottis. Evelina som spelar fiol i gruppen skrev låten till ett extra jobbigt stickningsprojekt som aldrig ville bli en färdig "Fusk Olle". Både du som spelat mycket förut eller inte spelat alls är välkommen att vara med! Lyssna på låten i förväg bland barnens låtar på sidan för Allspelslåtar.</t>
   </si>
 </sst>
 </file>
@@ -1088,7 +1094,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F23F1BC-D35E-3E42-8F88-5D61ED802479}">
-  <dimension ref="A1:Q84"/>
+  <dimension ref="A1:Q85"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.83203125" style="8" bestFit="1" customWidth="1"/>
@@ -3166,15 +3172,15 @@
         <v>114</v>
       </c>
     </row>
-    <row r="73" spans="1:17" ht="85" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:17" ht="119" x14ac:dyDescent="0.2">
       <c r="A73" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B73" s="9">
+        <v>0.625</v>
+      </c>
+      <c r="C73" s="9">
         <v>0.64583333333333337</v>
-      </c>
-      <c r="C73" s="9">
-        <v>0.66666666666666663</v>
       </c>
       <c r="D73" s="8" t="s">
         <v>41</v>
@@ -3186,24 +3192,24 @@
         <v>108</v>
       </c>
       <c r="H73" s="8" t="s">
-        <v>151</v>
+        <v>193</v>
       </c>
       <c r="I73" s="8">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="J73" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="74" spans="1:17" ht="34" x14ac:dyDescent="0.2">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="74" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A74" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B74" s="9">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="C74" s="9">
         <v>0.66666666666666663</v>
-      </c>
-      <c r="C74" s="9">
-        <v>0.6875</v>
       </c>
       <c r="D74" s="8" t="s">
         <v>41</v>
@@ -3215,115 +3221,118 @@
         <v>108</v>
       </c>
       <c r="H74" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="I74" s="8">
+        <v>58</v>
+      </c>
+      <c r="J74" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="75" spans="1:17" ht="34" x14ac:dyDescent="0.2">
+      <c r="A75" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B75" s="9">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C75" s="9">
+        <v>0.6875</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E75" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="F75" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="H75" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="I74" s="8">
+      <c r="I75" s="8">
         <v>59</v>
       </c>
-      <c r="J74" s="1" t="s">
+      <c r="J75" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="75" spans="1:17" ht="187" x14ac:dyDescent="0.2">
-      <c r="A75" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B75" s="9">
+    <row r="76" spans="1:17" ht="187" x14ac:dyDescent="0.2">
+      <c r="A76" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B76" s="9">
         <v>0.54166666666666663</v>
       </c>
-      <c r="C75" s="9">
+      <c r="C76" s="9">
         <v>0.58333333333333337</v>
       </c>
-      <c r="D75" s="8" t="s">
+      <c r="D76" s="8" t="s">
         <v>20</v>
-      </c>
-      <c r="E75" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F75" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="G75" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="H75" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="I75" s="8">
-        <v>60</v>
-      </c>
-      <c r="J75" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="L75" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="M75" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="N75" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="O75" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="P75" s="8" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q75" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="76" spans="1:17" ht="68" x14ac:dyDescent="0.2">
-      <c r="A76" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B76" s="9">
-        <v>0.9375</v>
-      </c>
-      <c r="C76" s="9">
-        <v>0</v>
-      </c>
-      <c r="D76" s="8" t="s">
-        <v>12</v>
       </c>
       <c r="E76" s="8" t="s">
         <v>25</v>
       </c>
+      <c r="F76" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="G76" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="H76" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="I76" s="8">
+        <v>60</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="L76" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="M76" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="N76" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="O76" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="P76" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q76" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17" ht="68" x14ac:dyDescent="0.2">
+      <c r="A77" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B77" s="9">
+        <v>0.9375</v>
+      </c>
+      <c r="C77" s="9">
+        <v>0</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E77" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="H77" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="I76" s="8">
+      <c r="I77" s="8">
         <v>61</v>
       </c>
-      <c r="J76" s="1" t="s">
+      <c r="J77" s="1" t="s">
         <v>116</v>
-      </c>
-    </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A77" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B77" s="9">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="C77" s="9">
-        <v>0.81944444444444442</v>
-      </c>
-      <c r="D77" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="E77" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="G77" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="H77" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="I77" s="8">
-        <v>62</v>
       </c>
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.2">
@@ -3331,10 +3340,10 @@
         <v>5</v>
       </c>
       <c r="B78" s="9">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C78" s="9">
         <v>0.81944444444444442</v>
-      </c>
-      <c r="C78" s="9">
-        <v>0.84722222222222221</v>
       </c>
       <c r="D78" s="8" t="s">
         <v>41</v>
@@ -3346,10 +3355,10 @@
         <v>33</v>
       </c>
       <c r="H78" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I78" s="8">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="79" spans="1:17" x14ac:dyDescent="0.2">
@@ -3357,10 +3366,10 @@
         <v>5</v>
       </c>
       <c r="B79" s="9">
+        <v>0.81944444444444442</v>
+      </c>
+      <c r="C79" s="9">
         <v>0.84722222222222221</v>
-      </c>
-      <c r="C79" s="9">
-        <v>0.875</v>
       </c>
       <c r="D79" s="8" t="s">
         <v>41</v>
@@ -3372,10 +3381,10 @@
         <v>33</v>
       </c>
       <c r="H79" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I79" s="8">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.2">
@@ -3383,10 +3392,10 @@
         <v>5</v>
       </c>
       <c r="B80" s="9">
+        <v>0.84722222222222221</v>
+      </c>
+      <c r="C80" s="9">
         <v>0.875</v>
-      </c>
-      <c r="C80" s="9">
-        <v>0.90277777777777779</v>
       </c>
       <c r="D80" s="8" t="s">
         <v>41</v>
@@ -3398,10 +3407,10 @@
         <v>33</v>
       </c>
       <c r="H80" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I80" s="8">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.2">
@@ -3409,10 +3418,10 @@
         <v>5</v>
       </c>
       <c r="B81" s="9">
+        <v>0.875</v>
+      </c>
+      <c r="C81" s="9">
         <v>0.90277777777777779</v>
-      </c>
-      <c r="C81" s="9">
-        <v>0.93055555555555558</v>
       </c>
       <c r="D81" s="8" t="s">
         <v>41</v>
@@ -3424,10 +3433,10 @@
         <v>33</v>
       </c>
       <c r="H81" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I81" s="8">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
@@ -3435,10 +3444,10 @@
         <v>5</v>
       </c>
       <c r="B82" s="9">
+        <v>0.90277777777777779</v>
+      </c>
+      <c r="C82" s="9">
         <v>0.93055555555555558</v>
-      </c>
-      <c r="C82" s="9">
-        <v>0.95833333333333337</v>
       </c>
       <c r="D82" s="8" t="s">
         <v>41</v>
@@ -3450,10 +3459,10 @@
         <v>33</v>
       </c>
       <c r="H82" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I82" s="8">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.2">
@@ -3461,10 +3470,10 @@
         <v>5</v>
       </c>
       <c r="B83" s="9">
+        <v>0.93055555555555558</v>
+      </c>
+      <c r="C83" s="9">
         <v>0.95833333333333337</v>
-      </c>
-      <c r="C83" s="9">
-        <v>0.98611111111111116</v>
       </c>
       <c r="D83" s="8" t="s">
         <v>41</v>
@@ -3476,10 +3485,10 @@
         <v>33</v>
       </c>
       <c r="H83" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I83" s="8">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.2">
@@ -3487,10 +3496,10 @@
         <v>5</v>
       </c>
       <c r="B84" s="9">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="C84" s="9">
         <v>0.98611111111111116</v>
-      </c>
-      <c r="C84" s="9">
-        <v>1.3888888888888888E-2</v>
       </c>
       <c r="D84" s="8" t="s">
         <v>41</v>
@@ -3502,9 +3511,35 @@
         <v>33</v>
       </c>
       <c r="H84" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="I84" s="8">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A85" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B85" s="9">
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="C85" s="9">
+        <v>1.3888888888888888E-2</v>
+      </c>
+      <c r="D85" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E85" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G85" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H85" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="I84" s="8">
+      <c r="I85" s="8">
         <v>69</v>
       </c>
     </row>

</xml_diff>